<commit_message>
chore: Inicializar estructura del monorepo y cargar documentacion base junto a readme
</commit_message>
<xml_diff>
--- a/docs/Diagramas_Actuales/Endpoints.xlsx
+++ b/docs/Diagramas_Actuales/Endpoints.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\agusp\OneDrive\Escritorio\UNLaM\Stock\Diagramas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\agusp\OneDrive\Escritorio\UNLaM\Proyecto_Stock_Fullstack\docs\Diagramas_Actuales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95C7C46A-3631-4CCC-B49A-8292DDB023EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC9867A4-3A31-4683-AFE6-7C5B9076B5F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00198741-A7AD-4B5A-8F84-9858E7D73BD8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="173">
   <si>
     <t>Metodo</t>
   </si>
@@ -553,6 +553,9 @@
   </si>
   <si>
     <t>JSON con los ingredientes de la receta, cantidades y rendimiento en unidades (kilos, cajas, etc)</t>
+  </si>
+  <si>
+    <t>Observaciones</t>
   </si>
 </sst>
 </file>
@@ -576,7 +579,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -584,32 +587,143 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -926,7 +1040,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99B52835-4C2D-409B-9707-A918CD91D2F1}">
-  <dimension ref="B10:K116"/>
+  <dimension ref="B9:K117"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="16.5703125" customWidth="1"/>
@@ -938,1825 +1052,2125 @@
     <col min="10" max="10" width="27.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
+    <row r="9" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H10" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="I10" t="s">
+      <c r="I10" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="J10" t="s">
+      <c r="J10" s="7" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B11" s="3" t="s">
+      <c r="K10" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G11" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="H11" t="s">
-        <v>13</v>
-      </c>
-      <c r="I11" t="s">
+      <c r="H11" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I11" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="J11" t="s">
+      <c r="J11" s="7" t="s">
         <v>16</v>
       </c>
       <c r="K11" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="G12" s="2"/>
-      <c r="I12" t="s">
+    <row r="12" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="J12" t="s">
+      <c r="J12" s="10" t="s">
         <v>18</v>
       </c>
       <c r="K12" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="G13" s="2"/>
-      <c r="I13" t="s">
+    <row r="13" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J13" t="s">
+      <c r="J13" s="10" t="s">
         <v>20</v>
       </c>
       <c r="K13" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="I14" t="s">
+    <row r="14" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="J14" t="s">
+      <c r="J14" s="17" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" t="s">
+    <row r="15" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="E15" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="G15" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="H15" t="s">
-        <v>13</v>
-      </c>
-      <c r="I15" t="s">
+      <c r="H15" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I15" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="J15" t="s">
+      <c r="J15" s="7" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" t="s">
+    <row r="16" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="10" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="G17" s="3"/>
-    </row>
-    <row r="18" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" t="s">
+      <c r="I16" s="10"/>
+      <c r="J16" s="10"/>
+    </row>
+    <row r="17" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="17"/>
+    </row>
+    <row r="18" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="E18" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G18" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="H18" t="s">
-        <v>13</v>
-      </c>
-      <c r="I18" t="s">
+      <c r="H18" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="I18" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="J18" t="s">
+      <c r="J18" s="10" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="I19" t="s">
+    <row r="19" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="J19" t="s">
+      <c r="J19" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="I20" t="s">
+    <row r="20" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="J20" t="s">
+      <c r="J20" s="10" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="21" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="I21" t="s">
+    <row r="21" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="17"/>
+      <c r="I21" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="J21" t="s">
+      <c r="J21" s="17" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B22" s="4" t="s">
+    <row r="22" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="E22" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="F22" s="2" t="s">
+      <c r="F22" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G22" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="H22" t="s">
-        <v>13</v>
-      </c>
-      <c r="I22" t="s">
+      <c r="H22" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I22" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="J22" t="s">
+      <c r="J22" s="7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B23" s="4"/>
-      <c r="C23" s="3"/>
-      <c r="F23" s="2"/>
-      <c r="I23" t="s">
+    <row r="23" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="6"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="J23" t="s">
+      <c r="J23" s="10" t="s">
         <v>18</v>
       </c>
       <c r="K23" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B24" s="4"/>
-      <c r="C24" s="3"/>
-      <c r="F24" s="2"/>
-    </row>
-    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B25" s="4"/>
-      <c r="C25" s="3"/>
-      <c r="I25" t="s">
+    <row r="24" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="6"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="10"/>
+      <c r="J24" s="10"/>
+    </row>
+    <row r="25" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="6"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="J25" t="s">
+      <c r="J25" s="17" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B26" s="4"/>
-      <c r="C26" s="3"/>
-      <c r="D26" t="s">
+    <row r="26" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="6"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="E26" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="F26" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="G26" t="s">
+      <c r="G26" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="H26" t="s">
-        <v>13</v>
-      </c>
-      <c r="I26" t="s">
+      <c r="H26" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="I26" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="J26" t="s">
+      <c r="J26" s="10" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="27" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B27" s="4"/>
-      <c r="C27" s="3"/>
-      <c r="F27" s="2"/>
-      <c r="I27" t="s">
+    <row r="27" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="6"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="J27" t="s">
+      <c r="J27" s="10" t="s">
         <v>18</v>
       </c>
       <c r="K27" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="28" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B28" s="4"/>
-      <c r="C28" s="3"/>
-      <c r="F28" s="2"/>
-    </row>
-    <row r="29" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B29" s="4"/>
-      <c r="C29" s="3"/>
-      <c r="I29" t="s">
+    <row r="28" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="6"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="12"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="10"/>
+      <c r="I28" s="10"/>
+      <c r="J28" s="10"/>
+    </row>
+    <row r="29" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="6"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="11"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="J29" t="s">
+      <c r="J29" s="10" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B30" s="4"/>
-      <c r="C30" s="3"/>
-      <c r="D30" t="s">
+    <row r="30" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="6"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="E30" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F30" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="G30" t="s">
+      <c r="G30" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="H30" t="s">
-        <v>13</v>
-      </c>
-      <c r="I30" t="s">
+      <c r="H30" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I30" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="J30" t="s">
+      <c r="J30" s="7" t="s">
         <v>16</v>
       </c>
       <c r="K30" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B31" s="4"/>
-      <c r="C31" s="3"/>
-      <c r="I31" t="s">
+    <row r="31" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="6"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="11"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="10"/>
+      <c r="H31" s="10"/>
+      <c r="I31" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="J31" t="s">
+      <c r="J31" s="10" t="s">
         <v>18</v>
       </c>
       <c r="K31" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="32" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B32" s="4"/>
-      <c r="C32" s="3"/>
-    </row>
-    <row r="33" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="4"/>
-      <c r="C33" s="3"/>
-      <c r="D33" t="s">
+    <row r="32" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="6"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="17"/>
+      <c r="H32" s="17"/>
+      <c r="I32" s="17"/>
+      <c r="J32" s="17"/>
+    </row>
+    <row r="33" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="6"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="E33" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="F33" t="s">
+      <c r="F33" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="G33" s="2" t="s">
+      <c r="G33" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="H33" t="s">
-        <v>13</v>
-      </c>
-      <c r="I33" t="s">
+      <c r="H33" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="I33" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="J33" t="s">
+      <c r="J33" s="10" t="s">
         <v>18</v>
       </c>
       <c r="K33" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B34" s="4"/>
-      <c r="C34" s="3"/>
-      <c r="G34" s="2"/>
-    </row>
-    <row r="35" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="4"/>
-      <c r="C35" s="3" t="s">
+    <row r="34" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="6"/>
+      <c r="C34" s="20"/>
+      <c r="D34" s="10"/>
+      <c r="E34" s="11"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="12"/>
+      <c r="H34" s="10"/>
+      <c r="I34" s="10"/>
+      <c r="J34" s="10"/>
+    </row>
+    <row r="35" spans="2:11" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="6"/>
+      <c r="C35" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D35" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="E35" s="1" t="s">
+      <c r="E35" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="F35" t="s">
+      <c r="F35" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="G35" s="2" t="s">
+      <c r="G35" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="H35" t="s">
-        <v>13</v>
-      </c>
-      <c r="I35" t="s">
+      <c r="H35" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I35" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="J35" t="s">
+      <c r="J35" s="7" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="36" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="4"/>
-      <c r="C36" s="3"/>
-      <c r="G36" s="2"/>
-    </row>
-    <row r="37" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B37" s="4"/>
-      <c r="C37" s="3"/>
-      <c r="G37" s="2"/>
+    <row r="36" spans="2:11" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B36" s="6"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="10"/>
+      <c r="G36" s="12"/>
+      <c r="H36" s="10"/>
+      <c r="I36" s="10"/>
+      <c r="J36" s="10"/>
+    </row>
+    <row r="37" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="6"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="18"/>
+      <c r="F37" s="17"/>
+      <c r="G37" s="19"/>
+      <c r="H37" s="17"/>
+      <c r="I37" s="17"/>
+      <c r="J37" s="17"/>
       <c r="K37" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="38" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="3" t="s">
+    <row r="38" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C38" s="3" t="s">
+      <c r="C38" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D38" t="s">
+      <c r="D38" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="E38" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="F38" t="s">
+      <c r="F38" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="G38" t="s">
+      <c r="G38" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="H38" t="s">
-        <v>13</v>
-      </c>
-      <c r="I38" t="s">
+      <c r="H38" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="I38" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="J38" t="s">
+      <c r="J38" s="10" t="s">
         <v>74</v>
       </c>
       <c r="K38" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="39" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B39" s="3"/>
-      <c r="C39" s="3"/>
-      <c r="I39" t="s">
+    <row r="39" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B39" s="4"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="11"/>
+      <c r="F39" s="10"/>
+      <c r="G39" s="10"/>
+      <c r="H39" s="10"/>
+      <c r="I39" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J39" t="s">
+      <c r="J39" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
-      <c r="I40" t="s">
+    <row r="40" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="4"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="11"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="I40" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="J40" t="s">
+      <c r="J40" s="10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="41" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B41" s="3"/>
-      <c r="C41" s="3"/>
-      <c r="I41" t="s">
+    <row r="41" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="11"/>
+      <c r="F41" s="10"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="I41" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="J41" t="s">
+      <c r="J41" s="10" t="s">
         <v>65</v>
       </c>
       <c r="K41" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B42" s="3"/>
-      <c r="C42" s="3"/>
-      <c r="I42" t="s">
+    <row r="42" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B42" s="4"/>
+      <c r="C42" s="4"/>
+      <c r="D42" s="10"/>
+      <c r="E42" s="11"/>
+      <c r="F42" s="10"/>
+      <c r="G42" s="10"/>
+      <c r="H42" s="10"/>
+      <c r="I42" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="J42" t="s">
+      <c r="J42" s="10" t="s">
         <v>75</v>
       </c>
       <c r="K42" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B43" s="3"/>
-      <c r="C43" s="3"/>
-      <c r="D43" t="s">
+    <row r="43" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B43" s="4"/>
+      <c r="C43" s="4"/>
+      <c r="D43" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E43" s="1" t="s">
+      <c r="E43" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="F43" t="s">
+      <c r="F43" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="G43" t="s">
+      <c r="G43" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="H43" t="s">
-        <v>13</v>
-      </c>
-      <c r="I43" t="s">
+      <c r="H43" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I43" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="J43" t="s">
+      <c r="J43" s="7" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="44" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B44" s="3"/>
-      <c r="C44" s="3"/>
-      <c r="E44" s="1" t="s">
+    <row r="44" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="10"/>
+      <c r="E44" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="I44" t="s">
+      <c r="F44" s="10"/>
+      <c r="G44" s="10"/>
+      <c r="H44" s="10"/>
+      <c r="I44" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="J44" t="s">
+      <c r="J44" s="10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="45" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B45" s="3"/>
-      <c r="C45" s="3"/>
-      <c r="I45" t="s">
+    <row r="45" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="17"/>
+      <c r="E45" s="18"/>
+      <c r="F45" s="17"/>
+      <c r="G45" s="17"/>
+      <c r="H45" s="17"/>
+      <c r="I45" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="J45" t="s">
+      <c r="J45" s="17" t="s">
         <v>65</v>
       </c>
       <c r="K45" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="46" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B46" s="3"/>
-      <c r="C46" s="3"/>
-      <c r="D46" t="s">
+    <row r="46" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B46" s="4"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E46" s="1" t="s">
+      <c r="E46" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="F46" t="s">
+      <c r="F46" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="G46" t="s">
+      <c r="G46" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="H46" t="s">
-        <v>13</v>
-      </c>
-      <c r="I46" t="s">
+      <c r="H46" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="I46" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J46" t="s">
+      <c r="J46" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="47" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B47" s="3"/>
-      <c r="C47" s="3"/>
-      <c r="E47" s="1" t="s">
+    <row r="47" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B47" s="4"/>
+      <c r="C47" s="4"/>
+      <c r="D47" s="10"/>
+      <c r="E47" s="11" t="s">
         <v>105</v>
       </c>
-      <c r="I47" t="s">
+      <c r="F47" s="10"/>
+      <c r="G47" s="10"/>
+      <c r="H47" s="10"/>
+      <c r="I47" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="J47" t="s">
+      <c r="J47" s="10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="48" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B48" s="3"/>
-      <c r="C48" s="3"/>
-      <c r="I48" t="s">
+    <row r="48" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B48" s="4"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="11"/>
+      <c r="F48" s="10"/>
+      <c r="G48" s="10"/>
+      <c r="H48" s="10"/>
+      <c r="I48" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="J48" t="s">
+      <c r="J48" s="10" t="s">
         <v>65</v>
       </c>
       <c r="K48" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="49" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B49" s="3"/>
-      <c r="C49" s="3"/>
-      <c r="D49" t="s">
+    <row r="49" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B49" s="4"/>
+      <c r="C49" s="4"/>
+      <c r="D49" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E49" s="1" t="s">
+      <c r="E49" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="F49" t="s">
+      <c r="F49" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="G49" t="s">
+      <c r="G49" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="H49" t="s">
-        <v>13</v>
-      </c>
-      <c r="I49" t="s">
+      <c r="H49" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I49" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="J49" t="s">
+      <c r="J49" s="7" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="50" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B50" s="3"/>
-      <c r="C50" s="3"/>
-      <c r="E50" s="1" t="s">
+    <row r="50" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B50" s="4"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="10"/>
+      <c r="E50" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="I50" t="s">
+      <c r="F50" s="10"/>
+      <c r="G50" s="10"/>
+      <c r="H50" s="10"/>
+      <c r="I50" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="J50" t="s">
+      <c r="J50" s="10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="51" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B51" s="3"/>
-      <c r="C51" s="3"/>
-      <c r="I51" t="s">
+    <row r="51" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B51" s="4"/>
+      <c r="C51" s="4"/>
+      <c r="D51" s="17"/>
+      <c r="E51" s="18"/>
+      <c r="F51" s="17"/>
+      <c r="G51" s="17"/>
+      <c r="H51" s="17"/>
+      <c r="I51" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="J51" t="s">
+      <c r="J51" s="17" t="s">
         <v>65</v>
       </c>
       <c r="K51" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="52" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B52" s="3"/>
-      <c r="C52" s="3"/>
-      <c r="D52" t="s">
+    <row r="52" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B52" s="4"/>
+      <c r="C52" s="4"/>
+      <c r="D52" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="E52" s="1" t="s">
+      <c r="E52" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="F52" t="s">
+      <c r="F52" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="G52" t="s">
+      <c r="G52" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="H52" t="s">
+      <c r="H52" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="I52" t="s">
+      <c r="I52" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="J52" t="s">
+      <c r="J52" s="10" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="53" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B53" s="3"/>
-      <c r="C53" s="3"/>
-      <c r="I53" t="s">
+    <row r="53" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B53" s="4"/>
+      <c r="C53" s="4"/>
+      <c r="D53" s="10"/>
+      <c r="E53" s="11"/>
+      <c r="F53" s="10"/>
+      <c r="G53" s="10"/>
+      <c r="H53" s="10"/>
+      <c r="I53" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J53" t="s">
+      <c r="J53" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="54" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B54" s="3"/>
-      <c r="C54" s="3"/>
-      <c r="I54" t="s">
+    <row r="54" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B54" s="4"/>
+      <c r="C54" s="4"/>
+      <c r="D54" s="10"/>
+      <c r="E54" s="11"/>
+      <c r="F54" s="10"/>
+      <c r="G54" s="10"/>
+      <c r="H54" s="10"/>
+      <c r="I54" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="J54" t="s">
+      <c r="J54" s="10" t="s">
         <v>29</v>
       </c>
       <c r="K54" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="55" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B55" s="3"/>
-      <c r="C55" s="3"/>
-      <c r="I55" t="s">
+    <row r="55" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B55" s="4"/>
+      <c r="C55" s="4"/>
+      <c r="D55" s="10"/>
+      <c r="E55" s="11"/>
+      <c r="F55" s="10"/>
+      <c r="G55" s="10"/>
+      <c r="H55" s="10"/>
+      <c r="I55" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="J55" t="s">
+      <c r="J55" s="10" t="s">
         <v>83</v>
       </c>
       <c r="K55" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="56" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B56" s="3"/>
-      <c r="C56" s="3" t="s">
+    <row r="56" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B56" s="4"/>
+      <c r="C56" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D56" t="s">
+      <c r="D56" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="E56" s="1" t="s">
+      <c r="E56" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="F56" s="2" t="s">
+      <c r="F56" s="22" t="s">
         <v>91</v>
       </c>
-      <c r="G56" s="2" t="s">
+      <c r="G56" s="22" t="s">
         <v>92</v>
       </c>
-      <c r="H56" t="s">
-        <v>13</v>
-      </c>
-      <c r="I56" t="s">
+      <c r="H56" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I56" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="J56" t="s">
+      <c r="J56" s="7" t="s">
         <v>93</v>
       </c>
       <c r="K56" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="57" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B57" s="3"/>
-      <c r="C57" s="3"/>
-      <c r="F57" s="2"/>
-      <c r="G57" s="2"/>
-      <c r="I57" t="s">
+    <row r="57" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B57" s="4"/>
+      <c r="C57" s="4"/>
+      <c r="D57" s="10"/>
+      <c r="E57" s="11"/>
+      <c r="F57" s="12"/>
+      <c r="G57" s="12"/>
+      <c r="H57" s="10"/>
+      <c r="I57" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J57" t="s">
+      <c r="J57" s="10" t="s">
         <v>79</v>
       </c>
       <c r="K57" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="58" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B58" s="3"/>
-      <c r="C58" s="3"/>
-      <c r="I58" t="s">
+    <row r="58" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B58" s="4"/>
+      <c r="C58" s="4"/>
+      <c r="D58" s="17"/>
+      <c r="E58" s="18"/>
+      <c r="F58" s="17"/>
+      <c r="G58" s="17"/>
+      <c r="H58" s="17"/>
+      <c r="I58" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="J58" t="s">
+      <c r="J58" s="17" t="s">
         <v>29</v>
       </c>
       <c r="K58" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="59" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B59" s="3"/>
-      <c r="C59" s="3"/>
-      <c r="D59" t="s">
+    <row r="59" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B59" s="4"/>
+      <c r="C59" s="4"/>
+      <c r="D59" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E59" s="1" t="s">
+      <c r="E59" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="F59" t="s">
+      <c r="F59" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="G59" t="s">
+      <c r="G59" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="H59" t="s">
-        <v>13</v>
-      </c>
-      <c r="I59" t="s">
+      <c r="H59" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="I59" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="J59" t="s">
+      <c r="J59" s="10" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="60" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B60" s="3"/>
-      <c r="C60" s="3"/>
-      <c r="I60" t="s">
+    <row r="60" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B60" s="4"/>
+      <c r="C60" s="4"/>
+      <c r="D60" s="10"/>
+      <c r="E60" s="11"/>
+      <c r="F60" s="10"/>
+      <c r="G60" s="10"/>
+      <c r="H60" s="10"/>
+      <c r="I60" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J60" t="s">
+      <c r="J60" s="10" t="s">
         <v>79</v>
       </c>
       <c r="K60" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="61" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B61" s="3"/>
-      <c r="C61" s="3"/>
-      <c r="D61" t="s">
+    <row r="61" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B61" s="4"/>
+      <c r="C61" s="4"/>
+      <c r="D61" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="E61" s="1" t="s">
+      <c r="E61" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="F61" t="s">
+      <c r="F61" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="G61" t="s">
+      <c r="G61" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="H61" t="s">
-        <v>13</v>
-      </c>
-      <c r="I61" t="s">
+      <c r="H61" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I61" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="J61" t="s">
+      <c r="J61" s="7" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="62" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B62" s="3"/>
-      <c r="C62" s="3"/>
-      <c r="I62" t="s">
+    <row r="62" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B62" s="4"/>
+      <c r="C62" s="4"/>
+      <c r="D62" s="17"/>
+      <c r="E62" s="18"/>
+      <c r="F62" s="17"/>
+      <c r="G62" s="17"/>
+      <c r="H62" s="17"/>
+      <c r="I62" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="J62" t="s">
+      <c r="J62" s="17" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="63" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B63" s="3"/>
-      <c r="C63" s="3"/>
-      <c r="D63" t="s">
+    <row r="63" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B63" s="4"/>
+      <c r="C63" s="4"/>
+      <c r="D63" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E63" s="5" t="s">
+      <c r="E63" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="F63" t="s">
+      <c r="F63" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="G63" t="s">
+      <c r="G63" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="H63" t="s">
-        <v>13</v>
-      </c>
-      <c r="I63" t="s">
+      <c r="H63" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="I63" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="J63" t="s">
+      <c r="J63" s="10" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="64" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B64" s="3"/>
-      <c r="C64" s="3"/>
-      <c r="E64" s="5"/>
-      <c r="I64" t="s">
+    <row r="64" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B64" s="4"/>
+      <c r="C64" s="4"/>
+      <c r="D64" s="10"/>
+      <c r="E64" s="13"/>
+      <c r="F64" s="10"/>
+      <c r="G64" s="10"/>
+      <c r="H64" s="10"/>
+      <c r="I64" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J64" t="s">
+      <c r="J64" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="65" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B65" s="3"/>
-      <c r="C65" s="3"/>
-      <c r="D65" t="s">
+    <row r="65" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B65" s="4"/>
+      <c r="C65" s="4"/>
+      <c r="D65" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E65" s="1" t="s">
+      <c r="E65" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="F65" t="s">
+      <c r="F65" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="G65" t="s">
+      <c r="G65" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="H65" t="s">
-        <v>13</v>
-      </c>
-      <c r="I65" t="s">
+      <c r="H65" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I65" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J65" t="s">
+      <c r="J65" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="66" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B66" s="3"/>
-      <c r="C66" s="3"/>
-      <c r="D66" t="s">
+    <row r="66" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B66" s="4"/>
+      <c r="C66" s="4"/>
+      <c r="D66" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E66" s="1" t="s">
+      <c r="E66" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="F66" t="s">
+      <c r="F66" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="G66" t="s">
+      <c r="G66" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="H66" t="s">
-        <v>13</v>
-      </c>
+      <c r="H66" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="I66" s="10"/>
+      <c r="J66" s="10"/>
       <c r="K66" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="67" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B67" s="3"/>
-      <c r="C67" s="3"/>
-      <c r="I67" t="s">
+    <row r="67" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B67" s="4"/>
+      <c r="C67" s="4"/>
+      <c r="D67" s="10"/>
+      <c r="E67" s="11"/>
+      <c r="F67" s="10"/>
+      <c r="G67" s="10"/>
+      <c r="H67" s="10"/>
+      <c r="I67" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J67" t="s">
+      <c r="J67" s="10" t="s">
         <v>79</v>
       </c>
       <c r="K67" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="68" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B68" s="3"/>
-      <c r="C68" s="3"/>
-      <c r="I68" t="s">
+    <row r="68" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B68" s="4"/>
+      <c r="C68" s="4"/>
+      <c r="D68" s="10"/>
+      <c r="E68" s="11"/>
+      <c r="F68" s="10"/>
+      <c r="G68" s="10"/>
+      <c r="H68" s="10"/>
+      <c r="I68" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="J68" t="s">
+      <c r="J68" s="10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="69" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B69" s="3"/>
-      <c r="C69" s="3"/>
-      <c r="D69" t="s">
+    <row r="69" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B69" s="4"/>
+      <c r="C69" s="4"/>
+      <c r="D69" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E69" s="1" t="s">
+      <c r="E69" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="F69" t="s">
+      <c r="F69" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="G69" t="s">
+      <c r="G69" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="H69" t="s">
-        <v>13</v>
-      </c>
-      <c r="I69" t="s">
+      <c r="H69" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I69" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="J69" t="s">
+      <c r="J69" s="7" t="s">
         <v>79</v>
       </c>
       <c r="K69" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="70" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B70" s="3"/>
-      <c r="C70" s="3"/>
-      <c r="E70" s="1" t="s">
+    <row r="70" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B70" s="4"/>
+      <c r="C70" s="4"/>
+      <c r="D70" s="17"/>
+      <c r="E70" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="I70" t="s">
+      <c r="F70" s="17"/>
+      <c r="G70" s="17"/>
+      <c r="H70" s="17"/>
+      <c r="I70" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="J70" t="s">
+      <c r="J70" s="17" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="71" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B71" s="3" t="s">
+    <row r="71" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B71" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="C71" s="3" t="s">
+      <c r="C71" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="D71" t="s">
+      <c r="D71" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="E71" s="1" t="s">
+      <c r="E71" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="F71" s="2" t="s">
+      <c r="F71" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="G71" t="s">
+      <c r="G71" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="H71" t="s">
+      <c r="H71" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="I71" t="s">
+      <c r="I71" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="J71" t="s">
+      <c r="J71" s="10" t="s">
         <v>74</v>
       </c>
       <c r="K71" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="72" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B72" s="3"/>
-      <c r="C72" s="3"/>
-      <c r="F72" s="2"/>
-      <c r="I72" t="s">
+    <row r="72" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B72" s="4"/>
+      <c r="C72" s="4"/>
+      <c r="D72" s="10"/>
+      <c r="E72" s="11"/>
+      <c r="F72" s="12"/>
+      <c r="G72" s="10"/>
+      <c r="H72" s="10"/>
+      <c r="I72" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J72" t="s">
+      <c r="J72" s="10" t="s">
         <v>79</v>
       </c>
       <c r="K72" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="73" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B73" s="3"/>
-      <c r="C73" s="3"/>
-      <c r="F73" s="2"/>
-      <c r="I73" t="s">
+    <row r="73" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B73" s="4"/>
+      <c r="C73" s="4"/>
+      <c r="D73" s="10"/>
+      <c r="E73" s="11"/>
+      <c r="F73" s="12"/>
+      <c r="G73" s="10"/>
+      <c r="H73" s="10"/>
+      <c r="I73" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="J73" t="s">
+      <c r="J73" s="10" t="s">
         <v>29</v>
       </c>
       <c r="K73" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="74" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B74" s="3"/>
-      <c r="C74" s="3"/>
-      <c r="D74" t="s">
+    <row r="74" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B74" s="4"/>
+      <c r="C74" s="4"/>
+      <c r="D74" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E74" s="1" t="s">
+      <c r="E74" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="F74" s="2" t="s">
+      <c r="F74" s="22" t="s">
         <v>125</v>
       </c>
-      <c r="G74" t="s">
+      <c r="G74" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="H74" t="s">
-        <v>13</v>
-      </c>
-      <c r="I74" t="s">
+      <c r="H74" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I74" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="J74" t="s">
+      <c r="J74" s="7" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="75" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B75" s="3"/>
-      <c r="C75" s="3"/>
-      <c r="F75" s="2"/>
-      <c r="I75" t="s">
+    <row r="75" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B75" s="4"/>
+      <c r="C75" s="4"/>
+      <c r="D75" s="10"/>
+      <c r="E75" s="11"/>
+      <c r="F75" s="12"/>
+      <c r="G75" s="10"/>
+      <c r="H75" s="10"/>
+      <c r="I75" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J75" t="s">
+      <c r="J75" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="76" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B76" s="3"/>
-      <c r="C76" s="3"/>
-      <c r="F76" s="2"/>
-      <c r="I76" t="s">
+    <row r="76" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B76" s="4"/>
+      <c r="C76" s="4"/>
+      <c r="D76" s="17"/>
+      <c r="E76" s="18"/>
+      <c r="F76" s="19"/>
+      <c r="G76" s="17"/>
+      <c r="H76" s="17"/>
+      <c r="I76" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="J76" t="s">
+      <c r="J76" s="17" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="77" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B77" s="3"/>
-      <c r="C77" s="2" t="s">
+    <row r="77" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B77" s="4"/>
+      <c r="C77" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="D77" t="s">
+      <c r="D77" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E77" s="5" t="s">
+      <c r="E77" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="F77" t="s">
+      <c r="F77" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="G77" s="2" t="s">
+      <c r="G77" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="H77" t="s">
-        <v>13</v>
-      </c>
-      <c r="I77" t="s">
+      <c r="H77" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="I77" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J77" t="s">
+      <c r="J77" s="10" t="s">
         <v>79</v>
       </c>
       <c r="K77" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="78" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B78" s="3"/>
-      <c r="C78" s="2"/>
-      <c r="E78" s="5"/>
-      <c r="G78" s="2"/>
-    </row>
-    <row r="79" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B79" s="3"/>
-      <c r="C79" s="2"/>
-      <c r="D79" t="s">
+    <row r="78" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B78" s="4"/>
+      <c r="C78" s="5"/>
+      <c r="D78" s="10"/>
+      <c r="E78" s="13"/>
+      <c r="F78" s="10"/>
+      <c r="G78" s="12"/>
+      <c r="H78" s="10"/>
+      <c r="I78" s="10"/>
+      <c r="J78" s="10"/>
+    </row>
+    <row r="79" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B79" s="4"/>
+      <c r="C79" s="5"/>
+      <c r="D79" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="E79" s="5" t="s">
+      <c r="E79" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="F79" t="s">
+      <c r="F79" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="G79" s="2" t="s">
+      <c r="G79" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="H79" t="s">
-        <v>13</v>
-      </c>
-      <c r="I79" t="s">
+      <c r="H79" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I79" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="J79" t="s">
+      <c r="J79" s="7" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="80" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B80" s="3"/>
-      <c r="C80" s="2"/>
-      <c r="E80" s="5"/>
-      <c r="G80" s="2"/>
-    </row>
-    <row r="81" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B81" s="4" t="s">
+    <row r="80" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B80" s="4"/>
+      <c r="C80" s="5"/>
+      <c r="D80" s="17"/>
+      <c r="E80" s="24"/>
+      <c r="F80" s="17"/>
+      <c r="G80" s="19"/>
+      <c r="H80" s="17"/>
+      <c r="I80" s="17"/>
+      <c r="J80" s="17"/>
+    </row>
+    <row r="81" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B81" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="C81" s="3" t="s">
+      <c r="C81" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D81" t="s">
+      <c r="D81" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="E81" s="1" t="s">
+      <c r="E81" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="F81" s="2" t="s">
+      <c r="F81" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="G81" t="s">
+      <c r="G81" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="H81" t="s">
+      <c r="H81" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="I81" t="s">
+      <c r="I81" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="J81" t="s">
+      <c r="J81" s="10" t="s">
         <v>74</v>
       </c>
       <c r="K81" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="82" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B82" s="4"/>
-      <c r="C82" s="3"/>
-      <c r="F82" s="2"/>
-      <c r="I82" t="s">
+    <row r="82" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B82" s="6"/>
+      <c r="C82" s="4"/>
+      <c r="D82" s="10"/>
+      <c r="E82" s="11"/>
+      <c r="F82" s="12"/>
+      <c r="G82" s="10"/>
+      <c r="H82" s="10"/>
+      <c r="I82" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J82" t="s">
+      <c r="J82" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="83" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B83" s="4"/>
-      <c r="C83" s="3"/>
-      <c r="D83" t="s">
+    <row r="83" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B83" s="6"/>
+      <c r="C83" s="4"/>
+      <c r="D83" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="E83" s="1" t="s">
+      <c r="E83" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="F83" s="7" t="s">
+      <c r="F83" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="G83" s="2" t="s">
+      <c r="G83" s="22" t="s">
         <v>131</v>
       </c>
-      <c r="H83" t="s">
-        <v>13</v>
-      </c>
-      <c r="I83" t="s">
+      <c r="H83" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I83" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="J83" t="s">
+      <c r="J83" s="7" t="s">
         <v>79</v>
       </c>
       <c r="K83" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="84" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B84" s="4"/>
-      <c r="C84" s="3"/>
-      <c r="E84" s="1" t="s">
+    <row r="84" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B84" s="6"/>
+      <c r="C84" s="4"/>
+      <c r="D84" s="17"/>
+      <c r="E84" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="F84" s="7"/>
-      <c r="G84" s="2"/>
-    </row>
-    <row r="85" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B85" s="4"/>
-      <c r="C85" s="3"/>
-      <c r="D85" t="s">
+      <c r="F84" s="26"/>
+      <c r="G84" s="19"/>
+      <c r="H84" s="17"/>
+      <c r="I84" s="17"/>
+      <c r="J84" s="17"/>
+    </row>
+    <row r="85" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B85" s="6"/>
+      <c r="C85" s="4"/>
+      <c r="D85" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E85" s="1" t="s">
+      <c r="E85" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="F85" t="s">
+      <c r="F85" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="G85" t="s">
+      <c r="G85" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="H85" t="s">
-        <v>13</v>
-      </c>
-      <c r="I85" t="s">
+      <c r="H85" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="I85" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J85" t="s">
+      <c r="J85" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="86" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B86" s="4"/>
-      <c r="C86" s="3"/>
-      <c r="I86" t="s">
+    <row r="86" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B86" s="6"/>
+      <c r="C86" s="4"/>
+      <c r="D86" s="10"/>
+      <c r="E86" s="11"/>
+      <c r="F86" s="10"/>
+      <c r="G86" s="10"/>
+      <c r="H86" s="10"/>
+      <c r="I86" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="J86" t="s">
+      <c r="J86" s="10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="87" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B87" s="4"/>
-      <c r="C87" s="3"/>
-      <c r="D87" t="s">
+    <row r="87" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B87" s="6"/>
+      <c r="C87" s="4"/>
+      <c r="D87" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E87" s="1" t="s">
+      <c r="E87" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="F87" t="s">
+      <c r="F87" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="G87" t="s">
+      <c r="G87" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="H87" t="s">
-        <v>13</v>
-      </c>
-      <c r="I87" t="s">
+      <c r="H87" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I87" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="J87" t="s">
+      <c r="J87" s="7" t="s">
         <v>79</v>
       </c>
       <c r="K87" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="88" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B88" s="4"/>
-      <c r="C88" s="3"/>
-      <c r="I88" t="s">
+    <row r="88" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B88" s="6"/>
+      <c r="C88" s="4"/>
+      <c r="D88" s="17"/>
+      <c r="E88" s="18"/>
+      <c r="F88" s="17"/>
+      <c r="G88" s="17"/>
+      <c r="H88" s="17"/>
+      <c r="I88" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="J88" t="s">
+      <c r="J88" s="17" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="89" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B89" s="4"/>
-      <c r="C89" s="3"/>
-      <c r="D89" t="s">
+    <row r="89" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B89" s="6"/>
+      <c r="C89" s="4"/>
+      <c r="D89" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E89" s="1" t="s">
+      <c r="E89" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="F89" t="s">
+      <c r="F89" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="G89" t="s">
+      <c r="G89" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="H89" t="s">
-        <v>13</v>
-      </c>
-      <c r="I89" t="s">
+      <c r="H89" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="I89" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="J89" t="s">
+      <c r="J89" s="10" t="s">
         <v>74</v>
       </c>
       <c r="K89" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="90" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B90" s="4"/>
-      <c r="C90" s="3"/>
-      <c r="I90" t="s">
+    <row r="90" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B90" s="6"/>
+      <c r="C90" s="4"/>
+      <c r="D90" s="10"/>
+      <c r="E90" s="11"/>
+      <c r="F90" s="10"/>
+      <c r="G90" s="10"/>
+      <c r="H90" s="10"/>
+      <c r="I90" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J90" t="s">
+      <c r="J90" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="91" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B91" s="4"/>
-      <c r="C91" s="3"/>
-      <c r="I91" t="s">
+    <row r="91" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B91" s="6"/>
+      <c r="C91" s="4"/>
+      <c r="D91" s="10"/>
+      <c r="E91" s="11"/>
+      <c r="F91" s="10"/>
+      <c r="G91" s="10"/>
+      <c r="H91" s="10"/>
+      <c r="I91" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="J91" t="s">
+      <c r="J91" s="10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="92" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B92" s="3" t="s">
+    <row r="92" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B92" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="C92" s="3" t="s">
+      <c r="C92" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="D92" t="s">
+      <c r="D92" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="E92" s="1" t="s">
+      <c r="E92" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="F92" t="s">
+      <c r="F92" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="G92" t="s">
+      <c r="G92" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="H92" t="s">
-        <v>13</v>
-      </c>
-      <c r="I92" t="s">
+      <c r="H92" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I92" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="J92" t="s">
+      <c r="J92" s="7" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="93" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B93" s="3"/>
-      <c r="C93" s="3"/>
-      <c r="I93" t="s">
+    <row r="93" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B93" s="4"/>
+      <c r="C93" s="4"/>
+      <c r="D93" s="17"/>
+      <c r="E93" s="18"/>
+      <c r="F93" s="17"/>
+      <c r="G93" s="17"/>
+      <c r="H93" s="17"/>
+      <c r="I93" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="J93" t="s">
+      <c r="J93" s="17" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="94" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B94" s="3"/>
-      <c r="C94" s="3"/>
-      <c r="D94" t="s">
+    <row r="94" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B94" s="4"/>
+      <c r="C94" s="4"/>
+      <c r="D94" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E94" s="5" t="s">
+      <c r="E94" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="F94" t="s">
+      <c r="F94" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="G94" s="2" t="s">
+      <c r="G94" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="H94" t="s">
-        <v>13</v>
-      </c>
-      <c r="I94" t="s">
+      <c r="H94" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="I94" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="J94" t="s">
+      <c r="J94" s="10" t="s">
         <v>70</v>
       </c>
       <c r="K94" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="95" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B95" s="3"/>
-      <c r="C95" s="3"/>
-      <c r="E95" s="5"/>
-      <c r="G95" s="2"/>
-      <c r="I95" t="s">
+    <row r="95" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B95" s="4"/>
+      <c r="C95" s="4"/>
+      <c r="D95" s="10"/>
+      <c r="E95" s="13"/>
+      <c r="F95" s="10"/>
+      <c r="G95" s="12"/>
+      <c r="H95" s="10"/>
+      <c r="I95" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J95" t="s">
+      <c r="J95" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="96" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B96" s="3"/>
-      <c r="C96" s="3"/>
-      <c r="E96" s="5"/>
-      <c r="G96" s="6"/>
+    <row r="96" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B96" s="4"/>
+      <c r="C96" s="4"/>
+      <c r="D96" s="10"/>
+      <c r="E96" s="13"/>
+      <c r="F96" s="10"/>
+      <c r="G96" s="14"/>
+      <c r="H96" s="10"/>
+      <c r="I96" s="10"/>
+      <c r="J96" s="10"/>
       <c r="K96" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="97" spans="2:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B97" s="3"/>
-      <c r="C97" s="3"/>
-      <c r="D97" t="s">
+    <row r="97" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B97" s="4"/>
+      <c r="C97" s="4"/>
+      <c r="D97" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="E97" s="8" t="s">
+      <c r="E97" s="27" t="s">
         <v>147</v>
       </c>
-      <c r="F97" t="s">
+      <c r="F97" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="G97" t="s">
+      <c r="G97" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="H97" t="s">
-        <v>13</v>
-      </c>
-      <c r="I97" t="s">
+      <c r="H97" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I97" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="J97" t="s">
+      <c r="J97" s="7" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="98" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B98" s="3"/>
-      <c r="C98" s="3"/>
-      <c r="E98" s="8"/>
-      <c r="I98" t="s">
+    <row r="98" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B98" s="4"/>
+      <c r="C98" s="4"/>
+      <c r="D98" s="10"/>
+      <c r="E98" s="15"/>
+      <c r="F98" s="10"/>
+      <c r="G98" s="10"/>
+      <c r="H98" s="10"/>
+      <c r="I98" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J98" t="s">
+      <c r="J98" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="99" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B99" s="3"/>
-      <c r="C99" s="3"/>
-      <c r="E99" s="8"/>
-      <c r="I99" t="s">
+    <row r="99" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B99" s="4"/>
+      <c r="C99" s="4"/>
+      <c r="D99" s="17"/>
+      <c r="E99" s="28"/>
+      <c r="F99" s="17"/>
+      <c r="G99" s="17"/>
+      <c r="H99" s="17"/>
+      <c r="I99" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="J99" t="s">
+      <c r="J99" s="17" t="s">
         <v>29</v>
       </c>
       <c r="K99" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="100" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B100" s="3" t="s">
+    <row r="100" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B100" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="C100" s="3" t="s">
+      <c r="C100" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="D100" t="s">
+      <c r="D100" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E100" s="1" t="s">
+      <c r="E100" s="11" t="s">
         <v>156</v>
       </c>
-      <c r="F100" t="s">
+      <c r="F100" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="G100" t="s">
+      <c r="G100" s="10" t="s">
         <v>158</v>
       </c>
-      <c r="H100" t="s">
-        <v>13</v>
-      </c>
-      <c r="I100" t="s">
+      <c r="H100" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="I100" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="J100" t="s">
+      <c r="J100" s="10" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="101" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B101" s="3"/>
-      <c r="C101" s="3"/>
-      <c r="I101" t="s">
+    <row r="101" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B101" s="4"/>
+      <c r="C101" s="4"/>
+      <c r="D101" s="10"/>
+      <c r="E101" s="11"/>
+      <c r="F101" s="10"/>
+      <c r="G101" s="10"/>
+      <c r="H101" s="10"/>
+      <c r="I101" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J101" t="s">
+      <c r="J101" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="102" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B102" s="3"/>
-      <c r="C102" s="3"/>
-      <c r="D102" t="s">
+    <row r="102" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B102" s="4"/>
+      <c r="C102" s="4"/>
+      <c r="D102" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="E102" s="1" t="s">
+      <c r="E102" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F102" t="s">
+      <c r="F102" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="G102" s="2" t="s">
+      <c r="G102" s="22" t="s">
         <v>159</v>
       </c>
-      <c r="H102" t="s">
-        <v>13</v>
-      </c>
-      <c r="I102" t="s">
+      <c r="H102" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I102" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="J102" t="s">
+      <c r="J102" s="7" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="103" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B103" s="3"/>
-      <c r="C103" s="3"/>
-      <c r="G103" s="2"/>
-      <c r="I103" t="s">
+    <row r="103" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B103" s="4"/>
+      <c r="C103" s="4"/>
+      <c r="D103" s="10"/>
+      <c r="E103" s="11"/>
+      <c r="F103" s="10"/>
+      <c r="G103" s="12"/>
+      <c r="H103" s="10"/>
+      <c r="I103" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J103" t="s">
+      <c r="J103" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="104" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B104" s="3"/>
-      <c r="C104" s="3"/>
-      <c r="I104" t="s">
+    <row r="104" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B104" s="4"/>
+      <c r="C104" s="4"/>
+      <c r="D104" s="17"/>
+      <c r="E104" s="18"/>
+      <c r="F104" s="17"/>
+      <c r="G104" s="17"/>
+      <c r="H104" s="17"/>
+      <c r="I104" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="J104" t="s">
+      <c r="J104" s="17" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="105" spans="2:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B105" s="3"/>
-      <c r="C105" s="3" t="s">
+    <row r="105" spans="2:11" ht="30" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B105" s="4"/>
+      <c r="C105" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D105" t="s">
+      <c r="D105" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="E105" s="1" t="s">
+      <c r="E105" s="11" t="s">
         <v>160</v>
       </c>
-      <c r="F105" s="3" t="s">
+      <c r="F105" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="G105" t="s">
+      <c r="G105" s="10" t="s">
         <v>161</v>
       </c>
-      <c r="H105" t="s">
+      <c r="H105" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="I105" t="s">
+      <c r="I105" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="J105" t="s">
+      <c r="J105" s="10" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="106" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B106" s="3"/>
-      <c r="C106" s="3"/>
-      <c r="F106" s="3"/>
-      <c r="I106" t="s">
+    <row r="106" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B106" s="4"/>
+      <c r="C106" s="4"/>
+      <c r="D106" s="10"/>
+      <c r="E106" s="11"/>
+      <c r="F106" s="9"/>
+      <c r="G106" s="10"/>
+      <c r="H106" s="10"/>
+      <c r="I106" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J106" t="s">
+      <c r="J106" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="107" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B107" s="3"/>
-      <c r="C107" s="3"/>
-      <c r="F107" s="3"/>
-      <c r="I107" t="s">
+    <row r="107" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B107" s="4"/>
+      <c r="C107" s="4"/>
+      <c r="D107" s="10"/>
+      <c r="E107" s="11"/>
+      <c r="F107" s="9"/>
+      <c r="G107" s="10"/>
+      <c r="H107" s="10"/>
+      <c r="I107" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="J107" t="s">
+      <c r="J107" s="10" t="s">
         <v>29</v>
       </c>
       <c r="K107" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="108" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B108" s="3"/>
-      <c r="C108" s="3"/>
-      <c r="D108" t="s">
+    <row r="108" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B108" s="4"/>
+      <c r="C108" s="4"/>
+      <c r="D108" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="E108" s="1" t="s">
+      <c r="E108" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F108" t="s">
+      <c r="F108" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="G108" t="s">
+      <c r="G108" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="H108" t="s">
-        <v>13</v>
-      </c>
-      <c r="I108" t="s">
+      <c r="H108" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I108" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="J108" t="s">
+      <c r="J108" s="7" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="109" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B109" s="3"/>
-      <c r="C109" s="3"/>
-      <c r="I109" t="s">
+    <row r="109" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B109" s="4"/>
+      <c r="C109" s="4"/>
+      <c r="D109" s="10"/>
+      <c r="E109" s="11"/>
+      <c r="F109" s="10"/>
+      <c r="G109" s="10"/>
+      <c r="H109" s="10"/>
+      <c r="I109" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="J109" t="s">
+      <c r="J109" s="10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="110" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B110" s="3"/>
-      <c r="C110" s="3"/>
-      <c r="I110" t="s">
+    <row r="110" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B110" s="4"/>
+      <c r="C110" s="4"/>
+      <c r="D110" s="17"/>
+      <c r="E110" s="18"/>
+      <c r="F110" s="17"/>
+      <c r="G110" s="17"/>
+      <c r="H110" s="17"/>
+      <c r="I110" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="J110" t="s">
+      <c r="J110" s="17" t="s">
         <v>163</v>
       </c>
       <c r="K110" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="111" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B111" s="3"/>
-      <c r="C111" s="3"/>
-      <c r="D111" t="s">
+    <row r="111" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B111" s="4"/>
+      <c r="C111" s="4"/>
+      <c r="D111" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E111" s="1" t="s">
+      <c r="E111" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="F111" t="s">
+      <c r="F111" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="G111" t="s">
+      <c r="G111" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="H111" t="s">
-        <v>13</v>
-      </c>
-      <c r="I111" t="s">
+      <c r="H111" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I111" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="J111" t="s">
+      <c r="J111" s="7" t="s">
         <v>74</v>
       </c>
       <c r="K111" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="112" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B112" s="3"/>
-      <c r="C112" s="3"/>
-      <c r="I112" t="s">
+    <row r="112" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B112" s="4"/>
+      <c r="C112" s="4"/>
+      <c r="D112" s="10"/>
+      <c r="E112" s="11"/>
+      <c r="F112" s="10"/>
+      <c r="G112" s="10"/>
+      <c r="H112" s="10"/>
+      <c r="I112" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J112" t="s">
+      <c r="J112" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="113" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B113" s="3"/>
-      <c r="C113" s="3"/>
-      <c r="I113" t="s">
+    <row r="113" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B113" s="4"/>
+      <c r="C113" s="4"/>
+      <c r="D113" s="10"/>
+      <c r="E113" s="11"/>
+      <c r="F113" s="10"/>
+      <c r="G113" s="10"/>
+      <c r="H113" s="10"/>
+      <c r="I113" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="J113" t="s">
+      <c r="J113" s="10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="114" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B114" s="3"/>
-      <c r="C114" s="3"/>
-      <c r="I114" t="s">
+    <row r="114" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B114" s="4"/>
+      <c r="C114" s="4"/>
+      <c r="D114" s="17"/>
+      <c r="E114" s="18"/>
+      <c r="F114" s="17"/>
+      <c r="G114" s="17"/>
+      <c r="H114" s="17"/>
+      <c r="I114" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="J114" t="s">
+      <c r="J114" s="17" t="s">
         <v>166</v>
       </c>
       <c r="K114" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="115" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B115" s="3"/>
-      <c r="C115" s="3"/>
-      <c r="D115" t="s">
+    <row r="115" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B115" s="4"/>
+      <c r="C115" s="4"/>
+      <c r="D115" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E115" s="1" t="s">
+      <c r="E115" s="11" t="s">
         <v>170</v>
       </c>
-      <c r="F115" s="2" t="s">
+      <c r="F115" s="12" t="s">
         <v>168</v>
       </c>
-      <c r="G115" t="s">
+      <c r="G115" s="10" t="s">
         <v>165</v>
       </c>
-      <c r="H115" t="s">
-        <v>13</v>
-      </c>
-      <c r="I115" t="s">
+      <c r="H115" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="I115" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="J115" t="s">
+      <c r="J115" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="116" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B116" s="3"/>
-      <c r="C116" s="3"/>
-      <c r="F116" s="2"/>
-      <c r="I116" t="s">
+    <row r="116" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B116" s="4"/>
+      <c r="C116" s="4"/>
+      <c r="D116" s="17"/>
+      <c r="E116" s="18"/>
+      <c r="F116" s="19"/>
+      <c r="G116" s="17"/>
+      <c r="H116" s="17"/>
+      <c r="I116" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="J116" t="s">
+      <c r="J116" s="17" t="s">
         <v>29</v>
       </c>
     </row>
+    <row r="117" spans="2:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="G102:G103"/>
-    <mergeCell ref="C105:C116"/>
-    <mergeCell ref="B100:B116"/>
-    <mergeCell ref="F105:F107"/>
-    <mergeCell ref="F115:F116"/>
-    <mergeCell ref="C92:C99"/>
-    <mergeCell ref="B92:B99"/>
-    <mergeCell ref="E94:E96"/>
-    <mergeCell ref="C100:C104"/>
-    <mergeCell ref="G83:G84"/>
-    <mergeCell ref="C81:C91"/>
-    <mergeCell ref="B81:B91"/>
-    <mergeCell ref="G94:G95"/>
-    <mergeCell ref="C77:C80"/>
-    <mergeCell ref="B71:B80"/>
-    <mergeCell ref="F74:F76"/>
-    <mergeCell ref="C71:C76"/>
-    <mergeCell ref="F81:F82"/>
-    <mergeCell ref="G35:G37"/>
-    <mergeCell ref="G33:G34"/>
-    <mergeCell ref="C22:C34"/>
-    <mergeCell ref="C35:C37"/>
-    <mergeCell ref="B38:B70"/>
-    <mergeCell ref="F71:F73"/>
-    <mergeCell ref="E77:E78"/>
-    <mergeCell ref="F56:F57"/>
-    <mergeCell ref="G56:G57"/>
-    <mergeCell ref="C38:C55"/>
-    <mergeCell ref="C56:C70"/>
-    <mergeCell ref="E79:E80"/>
     <mergeCell ref="G77:G78"/>
     <mergeCell ref="G79:G80"/>
     <mergeCell ref="B22:B37"/>
@@ -2767,6 +3181,36 @@
     <mergeCell ref="G15:G17"/>
     <mergeCell ref="C11:C21"/>
     <mergeCell ref="B11:B21"/>
+    <mergeCell ref="G35:G37"/>
+    <mergeCell ref="G33:G34"/>
+    <mergeCell ref="C22:C34"/>
+    <mergeCell ref="C35:C37"/>
+    <mergeCell ref="B38:B70"/>
+    <mergeCell ref="F56:F57"/>
+    <mergeCell ref="G56:G57"/>
+    <mergeCell ref="C38:C55"/>
+    <mergeCell ref="C56:C70"/>
+    <mergeCell ref="C77:C80"/>
+    <mergeCell ref="B71:B80"/>
+    <mergeCell ref="F74:F76"/>
+    <mergeCell ref="C71:C76"/>
+    <mergeCell ref="F81:F82"/>
+    <mergeCell ref="F71:F73"/>
+    <mergeCell ref="E77:E78"/>
+    <mergeCell ref="E79:E80"/>
+    <mergeCell ref="C92:C99"/>
+    <mergeCell ref="B92:B99"/>
+    <mergeCell ref="E94:E96"/>
+    <mergeCell ref="C100:C104"/>
+    <mergeCell ref="G83:G84"/>
+    <mergeCell ref="C81:C91"/>
+    <mergeCell ref="B81:B91"/>
+    <mergeCell ref="G94:G95"/>
+    <mergeCell ref="G102:G103"/>
+    <mergeCell ref="C105:C116"/>
+    <mergeCell ref="B100:B116"/>
+    <mergeCell ref="F105:F107"/>
+    <mergeCell ref="F115:F116"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
docs: agregar flujos de lotes (FEFO) y nuevos endpoints
</commit_message>
<xml_diff>
--- a/docs/Diagramas_Actuales/Endpoints.xlsx
+++ b/docs/Diagramas_Actuales/Endpoints.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\agusp\OneDrive\Escritorio\UNLaM\Proyecto_Stock_Fullstack\docs\Diagramas_Actuales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70808FC5-6AFA-44F3-A338-2A648484DC22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23E15A69-0EA1-4BEA-8BA8-3E8C298DE16F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00198741-A7AD-4B5A-8F84-9858E7D73BD8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="184">
   <si>
     <t>Metodo</t>
   </si>
@@ -556,6 +556,39 @@
   </si>
   <si>
     <t>compras?desde=dd-mm-yyyy&amp;hasta=dd-mm-yyyy&amp;ids=id1,id2&amp; idAutor=id1,id2</t>
+  </si>
+  <si>
+    <t>Lotes</t>
+  </si>
+  <si>
+    <t>lotes</t>
+  </si>
+  <si>
+    <t>JSON con los objetos Lote</t>
+  </si>
+  <si>
+    <t>lotes?idProducto=X&amp;estado=Y&amp;proximoAVencer=Z</t>
+  </si>
+  <si>
+    <t>Devuelve {} con params incorrectos</t>
+  </si>
+  <si>
+    <t>lotes/:id</t>
+  </si>
+  <si>
+    <t>JSON con el objeto Lote de id solicitado</t>
+  </si>
+  <si>
+    <t>JSON con el objeto Lote a crear</t>
+  </si>
+  <si>
+    <t>JSON con el objeto Lote creado</t>
+  </si>
+  <si>
+    <t>JSON con los datos modificados del lote</t>
+  </si>
+  <si>
+    <t>JSON con el objeto Lote modificado</t>
   </si>
 </sst>
 </file>
@@ -658,7 +691,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -687,38 +720,26 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -726,6 +747,22 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1040,7 +1077,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99B52835-4C2D-409B-9707-A918CD91D2F1}">
-  <dimension ref="B9:K118"/>
+  <dimension ref="B9:K129"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="16.5703125" customWidth="1"/>
@@ -1086,10 +1123,10 @@
       </c>
     </row>
     <row r="11" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="24" t="s">
+      <c r="B11" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="24" t="s">
+      <c r="C11" s="16" t="s">
         <v>57</v>
       </c>
       <c r="D11" s="4" t="s">
@@ -1101,7 +1138,7 @@
       <c r="F11" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G11" s="17" t="s">
+      <c r="G11" s="21" t="s">
         <v>21</v>
       </c>
       <c r="H11" s="4" t="s">
@@ -1118,12 +1155,12 @@
       </c>
     </row>
     <row r="12" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="24"/>
-      <c r="C12" s="24"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
       <c r="D12" s="6"/>
       <c r="E12" s="7"/>
       <c r="F12" s="6"/>
-      <c r="G12" s="16"/>
+      <c r="G12" s="18"/>
       <c r="H12" s="6"/>
       <c r="I12" s="6" t="s">
         <v>17</v>
@@ -1136,12 +1173,12 @@
       </c>
     </row>
     <row r="13" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="24"/>
-      <c r="C13" s="24"/>
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
       <c r="D13" s="6"/>
       <c r="E13" s="7"/>
       <c r="F13" s="6"/>
-      <c r="G13" s="16"/>
+      <c r="G13" s="18"/>
       <c r="H13" s="6"/>
       <c r="I13" s="6" t="s">
         <v>19</v>
@@ -1154,8 +1191,8 @@
       </c>
     </row>
     <row r="14" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="24"/>
-      <c r="C14" s="24"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="16"/>
       <c r="D14" s="10"/>
       <c r="E14" s="11"/>
       <c r="F14" s="10"/>
@@ -1169,8 +1206,8 @@
       </c>
     </row>
     <row r="15" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
       <c r="D15" s="4" t="s">
         <v>8</v>
       </c>
@@ -1180,7 +1217,7 @@
       <c r="F15" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="G15" s="21" t="s">
+      <c r="G15" s="26" t="s">
         <v>41</v>
       </c>
       <c r="H15" s="4" t="s">
@@ -1194,12 +1231,12 @@
       </c>
     </row>
     <row r="16" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="24"/>
-      <c r="C16" s="24"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
       <c r="D16" s="6"/>
       <c r="E16" s="7"/>
       <c r="F16" s="6"/>
-      <c r="G16" s="22"/>
+      <c r="G16" s="17"/>
       <c r="H16" s="6" t="s">
         <v>38</v>
       </c>
@@ -1207,19 +1244,19 @@
       <c r="J16" s="6"/>
     </row>
     <row r="17" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="24"/>
-      <c r="C17" s="24"/>
+      <c r="B17" s="16"/>
+      <c r="C17" s="16"/>
       <c r="D17" s="10"/>
       <c r="E17" s="11"/>
       <c r="F17" s="10"/>
-      <c r="G17" s="23"/>
+      <c r="G17" s="27"/>
       <c r="H17" s="10"/>
       <c r="I17" s="10"/>
       <c r="J17" s="10"/>
     </row>
     <row r="18" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
       <c r="D18" s="6" t="s">
         <v>8</v>
       </c>
@@ -1243,8 +1280,8 @@
       </c>
     </row>
     <row r="19" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
+      <c r="B19" s="16"/>
+      <c r="C19" s="16"/>
       <c r="D19" s="6"/>
       <c r="E19" s="7"/>
       <c r="F19" s="6"/>
@@ -1258,8 +1295,8 @@
       </c>
     </row>
     <row r="20" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="24"/>
-      <c r="C20" s="24"/>
+      <c r="B20" s="16"/>
+      <c r="C20" s="16"/>
       <c r="D20" s="6"/>
       <c r="E20" s="7"/>
       <c r="F20" s="6"/>
@@ -1273,8 +1310,8 @@
       </c>
     </row>
     <row r="21" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="24"/>
-      <c r="C21" s="24"/>
+      <c r="B21" s="16"/>
+      <c r="C21" s="16"/>
       <c r="D21" s="10"/>
       <c r="E21" s="11"/>
       <c r="F21" s="10"/>
@@ -1288,10 +1325,10 @@
       </c>
     </row>
     <row r="22" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="19" t="s">
+      <c r="B22" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="24" t="s">
+      <c r="C22" s="16" t="s">
         <v>58</v>
       </c>
       <c r="D22" s="4" t="s">
@@ -1300,7 +1337,7 @@
       <c r="E22" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="F22" s="17" t="s">
+      <c r="F22" s="21" t="s">
         <v>24</v>
       </c>
       <c r="G22" s="4" t="s">
@@ -1317,11 +1354,11 @@
       </c>
     </row>
     <row r="23" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="19"/>
-      <c r="C23" s="24"/>
+      <c r="B23" s="22"/>
+      <c r="C23" s="16"/>
       <c r="D23" s="6"/>
       <c r="E23" s="7"/>
-      <c r="F23" s="16"/>
+      <c r="F23" s="18"/>
       <c r="G23" s="6"/>
       <c r="H23" s="6"/>
       <c r="I23" s="6" t="s">
@@ -1335,19 +1372,19 @@
       </c>
     </row>
     <row r="24" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="19"/>
-      <c r="C24" s="24"/>
+      <c r="B24" s="22"/>
+      <c r="C24" s="16"/>
       <c r="D24" s="6"/>
       <c r="E24" s="7"/>
-      <c r="F24" s="16"/>
+      <c r="F24" s="18"/>
       <c r="G24" s="6"/>
       <c r="H24" s="6"/>
       <c r="I24" s="6"/>
       <c r="J24" s="6"/>
     </row>
     <row r="25" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="19"/>
-      <c r="C25" s="24"/>
+      <c r="B25" s="22"/>
+      <c r="C25" s="16"/>
       <c r="D25" s="10"/>
       <c r="E25" s="11"/>
       <c r="F25" s="10"/>
@@ -1361,15 +1398,15 @@
       </c>
     </row>
     <row r="26" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="19"/>
-      <c r="C26" s="24"/>
+      <c r="B26" s="22"/>
+      <c r="C26" s="16"/>
       <c r="D26" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="F26" s="16" t="s">
+      <c r="F26" s="18" t="s">
         <v>32</v>
       </c>
       <c r="G26" s="6" t="s">
@@ -1386,11 +1423,11 @@
       </c>
     </row>
     <row r="27" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="19"/>
-      <c r="C27" s="24"/>
+      <c r="B27" s="22"/>
+      <c r="C27" s="16"/>
       <c r="D27" s="6"/>
       <c r="E27" s="7"/>
-      <c r="F27" s="16"/>
+      <c r="F27" s="18"/>
       <c r="G27" s="6"/>
       <c r="H27" s="6"/>
       <c r="I27" s="6" t="s">
@@ -1404,19 +1441,19 @@
       </c>
     </row>
     <row r="28" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="19"/>
-      <c r="C28" s="24"/>
+      <c r="B28" s="22"/>
+      <c r="C28" s="16"/>
       <c r="D28" s="6"/>
       <c r="E28" s="7"/>
-      <c r="F28" s="16"/>
+      <c r="F28" s="18"/>
       <c r="G28" s="6"/>
       <c r="H28" s="6"/>
       <c r="I28" s="6"/>
       <c r="J28" s="6"/>
     </row>
     <row r="29" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="19"/>
-      <c r="C29" s="24"/>
+      <c r="B29" s="22"/>
+      <c r="C29" s="16"/>
       <c r="D29" s="6"/>
       <c r="E29" s="7"/>
       <c r="F29" s="6"/>
@@ -1430,8 +1467,8 @@
       </c>
     </row>
     <row r="30" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="19"/>
-      <c r="C30" s="24"/>
+      <c r="B30" s="22"/>
+      <c r="C30" s="16"/>
       <c r="D30" s="4" t="s">
         <v>9</v>
       </c>
@@ -1458,8 +1495,8 @@
       </c>
     </row>
     <row r="31" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="19"/>
-      <c r="C31" s="24"/>
+      <c r="B31" s="22"/>
+      <c r="C31" s="16"/>
       <c r="D31" s="6"/>
       <c r="E31" s="7"/>
       <c r="F31" s="6"/>
@@ -1476,8 +1513,8 @@
       </c>
     </row>
     <row r="32" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="19"/>
-      <c r="C32" s="24"/>
+      <c r="B32" s="22"/>
+      <c r="C32" s="16"/>
       <c r="D32" s="10"/>
       <c r="E32" s="11"/>
       <c r="F32" s="10"/>
@@ -1487,8 +1524,8 @@
       <c r="J32" s="10"/>
     </row>
     <row r="33" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="19"/>
-      <c r="C33" s="24"/>
+      <c r="B33" s="22"/>
+      <c r="C33" s="16"/>
       <c r="D33" s="6" t="s">
         <v>51</v>
       </c>
@@ -1498,7 +1535,7 @@
       <c r="F33" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="G33" s="16" t="s">
+      <c r="G33" s="18" t="s">
         <v>53</v>
       </c>
       <c r="H33" s="6" t="s">
@@ -1515,19 +1552,19 @@
       </c>
     </row>
     <row r="34" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="19"/>
-      <c r="C34" s="21"/>
+      <c r="B34" s="22"/>
+      <c r="C34" s="26"/>
       <c r="D34" s="6"/>
       <c r="E34" s="7"/>
       <c r="F34" s="6"/>
-      <c r="G34" s="16"/>
+      <c r="G34" s="18"/>
       <c r="H34" s="6"/>
       <c r="I34" s="6"/>
       <c r="J34" s="6"/>
     </row>
     <row r="35" spans="2:11" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="19"/>
-      <c r="C35" s="25" t="s">
+      <c r="B35" s="22"/>
+      <c r="C35" s="28" t="s">
         <v>88</v>
       </c>
       <c r="D35" s="4" t="s">
@@ -1539,7 +1576,7 @@
       <c r="F35" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="G35" s="17" t="s">
+      <c r="G35" s="21" t="s">
         <v>102</v>
       </c>
       <c r="H35" s="4" t="s">
@@ -1553,23 +1590,23 @@
       </c>
     </row>
     <row r="36" spans="2:11" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="19"/>
-      <c r="C36" s="24"/>
+      <c r="B36" s="22"/>
+      <c r="C36" s="16"/>
       <c r="D36" s="6"/>
       <c r="E36" s="7"/>
       <c r="F36" s="6"/>
-      <c r="G36" s="16"/>
+      <c r="G36" s="18"/>
       <c r="H36" s="6"/>
       <c r="I36" s="6"/>
       <c r="J36" s="6"/>
     </row>
     <row r="37" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="19"/>
-      <c r="C37" s="24"/>
+      <c r="B37" s="22"/>
+      <c r="C37" s="16"/>
       <c r="D37" s="10"/>
       <c r="E37" s="11"/>
       <c r="F37" s="10"/>
-      <c r="G37" s="18"/>
+      <c r="G37" s="19"/>
       <c r="H37" s="10"/>
       <c r="I37" s="10"/>
       <c r="J37" s="10"/>
@@ -1578,10 +1615,10 @@
       </c>
     </row>
     <row r="38" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="24" t="s">
+      <c r="B38" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="C38" s="24" t="s">
+      <c r="C38" s="16" t="s">
         <v>59</v>
       </c>
       <c r="D38" s="6" t="s">
@@ -1610,8 +1647,8 @@
       </c>
     </row>
     <row r="39" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="24"/>
-      <c r="C39" s="24"/>
+      <c r="B39" s="16"/>
+      <c r="C39" s="16"/>
       <c r="D39" s="6"/>
       <c r="E39" s="7"/>
       <c r="F39" s="6"/>
@@ -1625,8 +1662,8 @@
       </c>
     </row>
     <row r="40" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="24"/>
-      <c r="C40" s="24"/>
+      <c r="B40" s="16"/>
+      <c r="C40" s="16"/>
       <c r="D40" s="6"/>
       <c r="E40" s="7"/>
       <c r="F40" s="6"/>
@@ -1640,8 +1677,8 @@
       </c>
     </row>
     <row r="41" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="24"/>
-      <c r="C41" s="24"/>
+      <c r="B41" s="16"/>
+      <c r="C41" s="16"/>
       <c r="D41" s="6"/>
       <c r="E41" s="7"/>
       <c r="F41" s="6"/>
@@ -1658,8 +1695,8 @@
       </c>
     </row>
     <row r="42" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="24"/>
-      <c r="C42" s="24"/>
+      <c r="B42" s="16"/>
+      <c r="C42" s="16"/>
       <c r="D42" s="6"/>
       <c r="E42" s="7"/>
       <c r="F42" s="6"/>
@@ -1676,8 +1713,8 @@
       </c>
     </row>
     <row r="43" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="24"/>
-      <c r="C43" s="24"/>
+      <c r="B43" s="16"/>
+      <c r="C43" s="16"/>
       <c r="D43" s="4" t="s">
         <v>9</v>
       </c>
@@ -1701,8 +1738,8 @@
       </c>
     </row>
     <row r="44" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="24"/>
-      <c r="C44" s="24"/>
+      <c r="B44" s="16"/>
+      <c r="C44" s="16"/>
       <c r="D44" s="6"/>
       <c r="E44" s="7" t="s">
         <v>104</v>
@@ -1718,8 +1755,8 @@
       </c>
     </row>
     <row r="45" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="24"/>
-      <c r="C45" s="24"/>
+      <c r="B45" s="16"/>
+      <c r="C45" s="16"/>
       <c r="D45" s="10"/>
       <c r="E45" s="11"/>
       <c r="F45" s="10"/>
@@ -1736,8 +1773,8 @@
       </c>
     </row>
     <row r="46" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="24"/>
-      <c r="C46" s="24"/>
+      <c r="B46" s="16"/>
+      <c r="C46" s="16"/>
       <c r="D46" s="6" t="s">
         <v>9</v>
       </c>
@@ -1761,8 +1798,8 @@
       </c>
     </row>
     <row r="47" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="24"/>
-      <c r="C47" s="24"/>
+      <c r="B47" s="16"/>
+      <c r="C47" s="16"/>
       <c r="D47" s="6"/>
       <c r="E47" s="7" t="s">
         <v>105</v>
@@ -1778,8 +1815,8 @@
       </c>
     </row>
     <row r="48" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B48" s="24"/>
-      <c r="C48" s="24"/>
+      <c r="B48" s="16"/>
+      <c r="C48" s="16"/>
       <c r="D48" s="6"/>
       <c r="E48" s="7"/>
       <c r="F48" s="6"/>
@@ -1796,8 +1833,8 @@
       </c>
     </row>
     <row r="49" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="24"/>
-      <c r="C49" s="24"/>
+      <c r="B49" s="16"/>
+      <c r="C49" s="16"/>
       <c r="D49" s="4" t="s">
         <v>9</v>
       </c>
@@ -1821,8 +1858,8 @@
       </c>
     </row>
     <row r="50" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B50" s="24"/>
-      <c r="C50" s="24"/>
+      <c r="B50" s="16"/>
+      <c r="C50" s="16"/>
       <c r="D50" s="6"/>
       <c r="E50" s="7" t="s">
         <v>106</v>
@@ -1838,8 +1875,8 @@
       </c>
     </row>
     <row r="51" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B51" s="24"/>
-      <c r="C51" s="24"/>
+      <c r="B51" s="16"/>
+      <c r="C51" s="16"/>
       <c r="D51" s="10"/>
       <c r="E51" s="11"/>
       <c r="F51" s="10"/>
@@ -1856,8 +1893,8 @@
       </c>
     </row>
     <row r="52" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="24"/>
-      <c r="C52" s="24"/>
+      <c r="B52" s="16"/>
+      <c r="C52" s="16"/>
       <c r="D52" s="6" t="s">
         <v>8</v>
       </c>
@@ -1881,8 +1918,8 @@
       </c>
     </row>
     <row r="53" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B53" s="24"/>
-      <c r="C53" s="24"/>
+      <c r="B53" s="16"/>
+      <c r="C53" s="16"/>
       <c r="D53" s="6"/>
       <c r="E53" s="7"/>
       <c r="F53" s="6"/>
@@ -1896,8 +1933,8 @@
       </c>
     </row>
     <row r="54" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B54" s="24"/>
-      <c r="C54" s="24"/>
+      <c r="B54" s="16"/>
+      <c r="C54" s="16"/>
       <c r="D54" s="6"/>
       <c r="E54" s="7"/>
       <c r="F54" s="6"/>
@@ -1914,8 +1951,8 @@
       </c>
     </row>
     <row r="55" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="24"/>
-      <c r="C55" s="24"/>
+      <c r="B55" s="16"/>
+      <c r="C55" s="16"/>
       <c r="D55" s="6"/>
       <c r="E55" s="7"/>
       <c r="F55" s="6"/>
@@ -1932,8 +1969,8 @@
       </c>
     </row>
     <row r="56" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="24"/>
-      <c r="C56" s="24" t="s">
+      <c r="B56" s="16"/>
+      <c r="C56" s="16" t="s">
         <v>88</v>
       </c>
       <c r="D56" s="4" t="s">
@@ -1942,10 +1979,10 @@
       <c r="E56" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="F56" s="17" t="s">
+      <c r="F56" s="21" t="s">
         <v>91</v>
       </c>
-      <c r="G56" s="17" t="s">
+      <c r="G56" s="21" t="s">
         <v>92</v>
       </c>
       <c r="H56" s="4" t="s">
@@ -1962,12 +1999,12 @@
       </c>
     </row>
     <row r="57" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B57" s="24"/>
-      <c r="C57" s="24"/>
+      <c r="B57" s="16"/>
+      <c r="C57" s="16"/>
       <c r="D57" s="6"/>
       <c r="E57" s="7"/>
-      <c r="F57" s="16"/>
-      <c r="G57" s="16"/>
+      <c r="F57" s="18"/>
+      <c r="G57" s="18"/>
       <c r="H57" s="6"/>
       <c r="I57" s="6" t="s">
         <v>19</v>
@@ -1980,8 +2017,8 @@
       </c>
     </row>
     <row r="58" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B58" s="24"/>
-      <c r="C58" s="24"/>
+      <c r="B58" s="16"/>
+      <c r="C58" s="16"/>
       <c r="D58" s="10"/>
       <c r="E58" s="11"/>
       <c r="F58" s="10"/>
@@ -1998,8 +2035,8 @@
       </c>
     </row>
     <row r="59" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="24"/>
-      <c r="C59" s="24"/>
+      <c r="B59" s="16"/>
+      <c r="C59" s="16"/>
       <c r="D59" s="6" t="s">
         <v>51</v>
       </c>
@@ -2023,8 +2060,8 @@
       </c>
     </row>
     <row r="60" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="24"/>
-      <c r="C60" s="24"/>
+      <c r="B60" s="16"/>
+      <c r="C60" s="16"/>
       <c r="D60" s="6"/>
       <c r="E60" s="7"/>
       <c r="F60" s="6"/>
@@ -2041,8 +2078,8 @@
       </c>
     </row>
     <row r="61" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="24"/>
-      <c r="C61" s="24"/>
+      <c r="B61" s="16"/>
+      <c r="C61" s="16"/>
       <c r="D61" s="4" t="s">
         <v>51</v>
       </c>
@@ -2066,8 +2103,8 @@
       </c>
     </row>
     <row r="62" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B62" s="24"/>
-      <c r="C62" s="24"/>
+      <c r="B62" s="16"/>
+      <c r="C62" s="16"/>
       <c r="D62" s="10"/>
       <c r="E62" s="11"/>
       <c r="F62" s="10"/>
@@ -2081,8 +2118,8 @@
       </c>
     </row>
     <row r="63" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B63" s="24"/>
-      <c r="C63" s="24"/>
+      <c r="B63" s="16"/>
+      <c r="C63" s="16"/>
       <c r="D63" s="6" t="s">
         <v>51</v>
       </c>
@@ -2106,8 +2143,8 @@
       </c>
     </row>
     <row r="64" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="24"/>
-      <c r="C64" s="24"/>
+      <c r="B64" s="16"/>
+      <c r="C64" s="16"/>
       <c r="D64" s="6"/>
       <c r="E64" s="20"/>
       <c r="F64" s="6"/>
@@ -2121,8 +2158,8 @@
       </c>
     </row>
     <row r="65" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B65" s="24"/>
-      <c r="C65" s="24"/>
+      <c r="B65" s="16"/>
+      <c r="C65" s="16"/>
       <c r="D65" s="2" t="s">
         <v>51</v>
       </c>
@@ -2146,8 +2183,8 @@
       </c>
     </row>
     <row r="66" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B66" s="24"/>
-      <c r="C66" s="24"/>
+      <c r="B66" s="16"/>
+      <c r="C66" s="16"/>
       <c r="D66" s="6" t="s">
         <v>9</v>
       </c>
@@ -2170,8 +2207,8 @@
       </c>
     </row>
     <row r="67" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B67" s="24"/>
-      <c r="C67" s="24"/>
+      <c r="B67" s="16"/>
+      <c r="C67" s="16"/>
       <c r="D67" s="6"/>
       <c r="E67" s="7"/>
       <c r="F67" s="6"/>
@@ -2188,8 +2225,8 @@
       </c>
     </row>
     <row r="68" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B68" s="24"/>
-      <c r="C68" s="24"/>
+      <c r="B68" s="16"/>
+      <c r="C68" s="16"/>
       <c r="D68" s="6"/>
       <c r="E68" s="7"/>
       <c r="F68" s="6"/>
@@ -2203,8 +2240,8 @@
       </c>
     </row>
     <row r="69" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B69" s="24"/>
-      <c r="C69" s="24"/>
+      <c r="B69" s="16"/>
+      <c r="C69" s="16"/>
       <c r="D69" s="4" t="s">
         <v>9</v>
       </c>
@@ -2231,8 +2268,8 @@
       </c>
     </row>
     <row r="70" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B70" s="24"/>
-      <c r="C70" s="24"/>
+      <c r="B70" s="16"/>
+      <c r="C70" s="16"/>
       <c r="D70" s="10"/>
       <c r="E70" s="11" t="s">
         <v>106</v>
@@ -2248,10 +2285,10 @@
       </c>
     </row>
     <row r="71" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B71" s="24" t="s">
+      <c r="B71" s="16" t="s">
         <v>110</v>
       </c>
-      <c r="C71" s="24" t="s">
+      <c r="C71" s="16" t="s">
         <v>121</v>
       </c>
       <c r="D71" s="6" t="s">
@@ -2260,7 +2297,7 @@
       <c r="E71" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="F71" s="16" t="s">
+      <c r="F71" s="18" t="s">
         <v>115</v>
       </c>
       <c r="G71" s="6" t="s">
@@ -2280,11 +2317,11 @@
       </c>
     </row>
     <row r="72" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B72" s="24"/>
-      <c r="C72" s="24"/>
+      <c r="B72" s="16"/>
+      <c r="C72" s="16"/>
       <c r="D72" s="6"/>
       <c r="E72" s="7"/>
-      <c r="F72" s="16"/>
+      <c r="F72" s="18"/>
       <c r="G72" s="6"/>
       <c r="H72" s="6"/>
       <c r="I72" s="6" t="s">
@@ -2298,11 +2335,11 @@
       </c>
     </row>
     <row r="73" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B73" s="24"/>
-      <c r="C73" s="24"/>
+      <c r="B73" s="16"/>
+      <c r="C73" s="16"/>
       <c r="D73" s="6"/>
       <c r="E73" s="7"/>
-      <c r="F73" s="16"/>
+      <c r="F73" s="18"/>
       <c r="G73" s="6"/>
       <c r="H73" s="6"/>
       <c r="I73" s="6" t="s">
@@ -2316,15 +2353,15 @@
       </c>
     </row>
     <row r="74" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B74" s="24"/>
-      <c r="C74" s="24"/>
+      <c r="B74" s="16"/>
+      <c r="C74" s="16"/>
       <c r="D74" s="4" t="s">
         <v>9</v>
       </c>
       <c r="E74" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="F74" s="17" t="s">
+      <c r="F74" s="21" t="s">
         <v>124</v>
       </c>
       <c r="G74" s="4" t="s">
@@ -2341,11 +2378,11 @@
       </c>
     </row>
     <row r="75" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B75" s="24"/>
-      <c r="C75" s="24"/>
+      <c r="B75" s="16"/>
+      <c r="C75" s="16"/>
       <c r="D75" s="6"/>
       <c r="E75" s="7"/>
-      <c r="F75" s="16"/>
+      <c r="F75" s="18"/>
       <c r="G75" s="6"/>
       <c r="H75" s="6"/>
       <c r="I75" s="6" t="s">
@@ -2356,11 +2393,11 @@
       </c>
     </row>
     <row r="76" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B76" s="24"/>
-      <c r="C76" s="24"/>
+      <c r="B76" s="16"/>
+      <c r="C76" s="16"/>
       <c r="D76" s="10"/>
       <c r="E76" s="11"/>
-      <c r="F76" s="18"/>
+      <c r="F76" s="19"/>
       <c r="G76" s="10"/>
       <c r="H76" s="10"/>
       <c r="I76" s="10" t="s">
@@ -2371,8 +2408,8 @@
       </c>
     </row>
     <row r="77" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B77" s="24"/>
-      <c r="C77" s="26" t="s">
+      <c r="B77" s="16"/>
+      <c r="C77" s="25" t="s">
         <v>122</v>
       </c>
       <c r="D77" s="6" t="s">
@@ -2384,7 +2421,7 @@
       <c r="F77" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="G77" s="16" t="s">
+      <c r="G77" s="18" t="s">
         <v>119</v>
       </c>
       <c r="H77" s="6" t="s">
@@ -2401,40 +2438,40 @@
       </c>
     </row>
     <row r="78" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B78" s="24"/>
-      <c r="C78" s="26"/>
+      <c r="B78" s="16"/>
+      <c r="C78" s="25"/>
       <c r="D78" s="6"/>
       <c r="E78" s="20"/>
       <c r="F78" s="6"/>
-      <c r="G78" s="16"/>
+      <c r="G78" s="18"/>
       <c r="H78" s="6"/>
       <c r="I78" s="6"/>
       <c r="J78" s="6"/>
     </row>
     <row r="79" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B79" s="24"/>
-      <c r="C79" s="26"/>
+      <c r="B79" s="16"/>
+      <c r="C79" s="25"/>
       <c r="D79" s="6"/>
       <c r="E79" s="20"/>
       <c r="F79" s="6"/>
-      <c r="G79" s="16"/>
+      <c r="G79" s="18"/>
       <c r="H79" s="6"/>
       <c r="I79" s="6"/>
       <c r="J79" s="6"/>
     </row>
     <row r="80" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B80" s="24"/>
-      <c r="C80" s="26"/>
+      <c r="B80" s="16"/>
+      <c r="C80" s="25"/>
       <c r="D80" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="E80" s="27" t="s">
+      <c r="E80" s="23" t="s">
         <v>118</v>
       </c>
       <c r="F80" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="G80" s="17" t="s">
+      <c r="G80" s="21" t="s">
         <v>120</v>
       </c>
       <c r="H80" s="4" t="s">
@@ -2448,21 +2485,21 @@
       </c>
     </row>
     <row r="81" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B81" s="24"/>
-      <c r="C81" s="26"/>
+      <c r="B81" s="16"/>
+      <c r="C81" s="25"/>
       <c r="D81" s="10"/>
-      <c r="E81" s="28"/>
+      <c r="E81" s="24"/>
       <c r="F81" s="10"/>
-      <c r="G81" s="18"/>
+      <c r="G81" s="19"/>
       <c r="H81" s="10"/>
       <c r="I81" s="10"/>
       <c r="J81" s="10"/>
     </row>
     <row r="82" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B82" s="19" t="s">
+      <c r="B82" s="22" t="s">
         <v>137</v>
       </c>
-      <c r="C82" s="24" t="s">
+      <c r="C82" s="16" t="s">
         <v>88</v>
       </c>
       <c r="D82" s="6" t="s">
@@ -2471,7 +2508,7 @@
       <c r="E82" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="F82" s="16" t="s">
+      <c r="F82" s="18" t="s">
         <v>127</v>
       </c>
       <c r="G82" s="6" t="s">
@@ -2491,11 +2528,11 @@
       </c>
     </row>
     <row r="83" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B83" s="19"/>
-      <c r="C83" s="24"/>
+      <c r="B83" s="22"/>
+      <c r="C83" s="16"/>
       <c r="D83" s="6"/>
       <c r="E83" s="7"/>
-      <c r="F83" s="16"/>
+      <c r="F83" s="18"/>
       <c r="G83" s="6"/>
       <c r="H83" s="6"/>
       <c r="I83" s="6" t="s">
@@ -2506,8 +2543,8 @@
       </c>
     </row>
     <row r="84" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B84" s="19"/>
-      <c r="C84" s="24"/>
+      <c r="B84" s="22"/>
+      <c r="C84" s="16"/>
       <c r="D84" s="4" t="s">
         <v>51</v>
       </c>
@@ -2517,7 +2554,7 @@
       <c r="F84" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="G84" s="17" t="s">
+      <c r="G84" s="21" t="s">
         <v>130</v>
       </c>
       <c r="H84" s="4" t="s">
@@ -2534,21 +2571,21 @@
       </c>
     </row>
     <row r="85" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B85" s="19"/>
-      <c r="C85" s="24"/>
+      <c r="B85" s="22"/>
+      <c r="C85" s="16"/>
       <c r="D85" s="10"/>
       <c r="E85" s="11" t="s">
         <v>132</v>
       </c>
       <c r="F85" s="13"/>
-      <c r="G85" s="18"/>
+      <c r="G85" s="19"/>
       <c r="H85" s="10"/>
       <c r="I85" s="10"/>
       <c r="J85" s="10"/>
     </row>
     <row r="86" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B86" s="19"/>
-      <c r="C86" s="24"/>
+      <c r="B86" s="22"/>
+      <c r="C86" s="16"/>
       <c r="D86" s="6" t="s">
         <v>51</v>
       </c>
@@ -2572,8 +2609,8 @@
       </c>
     </row>
     <row r="87" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B87" s="19"/>
-      <c r="C87" s="24"/>
+      <c r="B87" s="22"/>
+      <c r="C87" s="16"/>
       <c r="D87" s="6"/>
       <c r="E87" s="7"/>
       <c r="F87" s="6"/>
@@ -2587,8 +2624,8 @@
       </c>
     </row>
     <row r="88" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B88" s="19"/>
-      <c r="C88" s="24"/>
+      <c r="B88" s="22"/>
+      <c r="C88" s="16"/>
       <c r="D88" s="4" t="s">
         <v>9</v>
       </c>
@@ -2615,8 +2652,8 @@
       </c>
     </row>
     <row r="89" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B89" s="19"/>
-      <c r="C89" s="24"/>
+      <c r="B89" s="22"/>
+      <c r="C89" s="16"/>
       <c r="D89" s="10"/>
       <c r="E89" s="11"/>
       <c r="F89" s="10"/>
@@ -2630,8 +2667,8 @@
       </c>
     </row>
     <row r="90" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B90" s="19"/>
-      <c r="C90" s="24"/>
+      <c r="B90" s="22"/>
+      <c r="C90" s="16"/>
       <c r="D90" s="6" t="s">
         <v>9</v>
       </c>
@@ -2658,8 +2695,8 @@
       </c>
     </row>
     <row r="91" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B91" s="19"/>
-      <c r="C91" s="24"/>
+      <c r="B91" s="22"/>
+      <c r="C91" s="16"/>
       <c r="D91" s="6"/>
       <c r="E91" s="7"/>
       <c r="F91" s="6"/>
@@ -2673,8 +2710,8 @@
       </c>
     </row>
     <row r="92" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B92" s="19"/>
-      <c r="C92" s="24"/>
+      <c r="B92" s="22"/>
+      <c r="C92" s="16"/>
       <c r="D92" s="6"/>
       <c r="E92" s="7"/>
       <c r="F92" s="6"/>
@@ -2688,10 +2725,10 @@
       </c>
     </row>
     <row r="93" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B93" s="24" t="s">
+      <c r="B93" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="C93" s="24" t="s">
+      <c r="C93" s="16" t="s">
         <v>122</v>
       </c>
       <c r="D93" s="4" t="s">
@@ -2717,8 +2754,8 @@
       </c>
     </row>
     <row r="94" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B94" s="24"/>
-      <c r="C94" s="24"/>
+      <c r="B94" s="16"/>
+      <c r="C94" s="16"/>
       <c r="D94" s="10"/>
       <c r="E94" s="11"/>
       <c r="F94" s="10"/>
@@ -2732,8 +2769,8 @@
       </c>
     </row>
     <row r="95" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B95" s="24"/>
-      <c r="C95" s="24"/>
+      <c r="B95" s="16"/>
+      <c r="C95" s="16"/>
       <c r="D95" s="6" t="s">
         <v>51</v>
       </c>
@@ -2743,7 +2780,7 @@
       <c r="F95" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="G95" s="16" t="s">
+      <c r="G95" s="18" t="s">
         <v>150</v>
       </c>
       <c r="H95" s="6" t="s">
@@ -2760,12 +2797,12 @@
       </c>
     </row>
     <row r="96" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B96" s="24"/>
-      <c r="C96" s="24"/>
+      <c r="B96" s="16"/>
+      <c r="C96" s="16"/>
       <c r="D96" s="6"/>
       <c r="E96" s="20"/>
       <c r="F96" s="6"/>
-      <c r="G96" s="16"/>
+      <c r="G96" s="18"/>
       <c r="H96" s="6"/>
       <c r="I96" s="6" t="s">
         <v>19</v>
@@ -2775,8 +2812,8 @@
       </c>
     </row>
     <row r="97" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B97" s="24"/>
-      <c r="C97" s="24"/>
+      <c r="B97" s="16"/>
+      <c r="C97" s="16"/>
       <c r="D97" s="6"/>
       <c r="E97" s="20"/>
       <c r="F97" s="6"/>
@@ -2789,8 +2826,8 @@
       </c>
     </row>
     <row r="98" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B98" s="24"/>
-      <c r="C98" s="24"/>
+      <c r="B98" s="16"/>
+      <c r="C98" s="16"/>
       <c r="D98" s="4" t="s">
         <v>51</v>
       </c>
@@ -2814,8 +2851,8 @@
       </c>
     </row>
     <row r="99" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B99" s="24"/>
-      <c r="C99" s="24"/>
+      <c r="B99" s="16"/>
+      <c r="C99" s="16"/>
       <c r="D99" s="6"/>
       <c r="E99" s="9"/>
       <c r="F99" s="6"/>
@@ -2829,8 +2866,8 @@
       </c>
     </row>
     <row r="100" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B100" s="24"/>
-      <c r="C100" s="24"/>
+      <c r="B100" s="16"/>
+      <c r="C100" s="16"/>
       <c r="D100" s="10"/>
       <c r="E100" s="15"/>
       <c r="F100" s="10"/>
@@ -2847,10 +2884,10 @@
       </c>
     </row>
     <row r="101" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B101" s="24" t="s">
+      <c r="B101" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="C101" s="24" t="s">
+      <c r="C101" s="16" t="s">
         <v>154</v>
       </c>
       <c r="D101" s="6" t="s">
@@ -2876,8 +2913,8 @@
       </c>
     </row>
     <row r="102" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B102" s="24"/>
-      <c r="C102" s="24"/>
+      <c r="B102" s="16"/>
+      <c r="C102" s="16"/>
       <c r="D102" s="6"/>
       <c r="E102" s="7"/>
       <c r="F102" s="6"/>
@@ -2891,8 +2928,8 @@
       </c>
     </row>
     <row r="103" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B103" s="24"/>
-      <c r="C103" s="24"/>
+      <c r="B103" s="16"/>
+      <c r="C103" s="16"/>
       <c r="D103" s="4" t="s">
         <v>51</v>
       </c>
@@ -2902,7 +2939,7 @@
       <c r="F103" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="G103" s="17" t="s">
+      <c r="G103" s="21" t="s">
         <v>158</v>
       </c>
       <c r="H103" s="4" t="s">
@@ -2916,12 +2953,12 @@
       </c>
     </row>
     <row r="104" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B104" s="24"/>
-      <c r="C104" s="24"/>
+      <c r="B104" s="16"/>
+      <c r="C104" s="16"/>
       <c r="D104" s="6"/>
       <c r="E104" s="7"/>
       <c r="F104" s="6"/>
-      <c r="G104" s="16"/>
+      <c r="G104" s="18"/>
       <c r="H104" s="6"/>
       <c r="I104" s="6" t="s">
         <v>19</v>
@@ -2931,8 +2968,8 @@
       </c>
     </row>
     <row r="105" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B105" s="24"/>
-      <c r="C105" s="24"/>
+      <c r="B105" s="16"/>
+      <c r="C105" s="16"/>
       <c r="D105" s="10"/>
       <c r="E105" s="11"/>
       <c r="F105" s="10"/>
@@ -2946,8 +2983,8 @@
       </c>
     </row>
     <row r="106" spans="2:11" ht="30" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B106" s="24"/>
-      <c r="C106" s="24" t="s">
+      <c r="B106" s="16"/>
+      <c r="C106" s="16" t="s">
         <v>59</v>
       </c>
       <c r="D106" s="6" t="s">
@@ -2956,7 +2993,7 @@
       <c r="E106" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="F106" s="22" t="s">
+      <c r="F106" s="17" t="s">
         <v>170</v>
       </c>
       <c r="G106" s="6" t="s">
@@ -2973,11 +3010,11 @@
       </c>
     </row>
     <row r="107" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B107" s="24"/>
-      <c r="C107" s="24"/>
+      <c r="B107" s="16"/>
+      <c r="C107" s="16"/>
       <c r="D107" s="6"/>
       <c r="E107" s="7"/>
-      <c r="F107" s="22"/>
+      <c r="F107" s="17"/>
       <c r="G107" s="6"/>
       <c r="H107" s="6"/>
       <c r="I107" s="6" t="s">
@@ -2988,11 +3025,11 @@
       </c>
     </row>
     <row r="108" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B108" s="24"/>
-      <c r="C108" s="24"/>
+      <c r="B108" s="16"/>
+      <c r="C108" s="16"/>
       <c r="D108" s="6"/>
       <c r="E108" s="7"/>
-      <c r="F108" s="22"/>
+      <c r="F108" s="17"/>
       <c r="G108" s="6"/>
       <c r="H108" s="6"/>
       <c r="I108" s="6" t="s">
@@ -3006,8 +3043,8 @@
       </c>
     </row>
     <row r="109" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B109" s="24"/>
-      <c r="C109" s="24"/>
+      <c r="B109" s="16"/>
+      <c r="C109" s="16"/>
       <c r="D109" s="4" t="s">
         <v>85</v>
       </c>
@@ -3031,8 +3068,8 @@
       </c>
     </row>
     <row r="110" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B110" s="24"/>
-      <c r="C110" s="24"/>
+      <c r="B110" s="16"/>
+      <c r="C110" s="16"/>
       <c r="D110" s="6"/>
       <c r="E110" s="7"/>
       <c r="F110" s="6"/>
@@ -3046,8 +3083,8 @@
       </c>
     </row>
     <row r="111" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B111" s="24"/>
-      <c r="C111" s="24"/>
+      <c r="B111" s="16"/>
+      <c r="C111" s="16"/>
       <c r="D111" s="10"/>
       <c r="E111" s="11"/>
       <c r="F111" s="10"/>
@@ -3064,8 +3101,8 @@
       </c>
     </row>
     <row r="112" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B112" s="24"/>
-      <c r="C112" s="24"/>
+      <c r="B112" s="16"/>
+      <c r="C112" s="16"/>
       <c r="D112" s="4" t="s">
         <v>9</v>
       </c>
@@ -3092,8 +3129,8 @@
       </c>
     </row>
     <row r="113" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B113" s="24"/>
-      <c r="C113" s="24"/>
+      <c r="B113" s="16"/>
+      <c r="C113" s="16"/>
       <c r="D113" s="6"/>
       <c r="E113" s="7"/>
       <c r="F113" s="6"/>
@@ -3107,8 +3144,8 @@
       </c>
     </row>
     <row r="114" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B114" s="24"/>
-      <c r="C114" s="24"/>
+      <c r="B114" s="16"/>
+      <c r="C114" s="16"/>
       <c r="D114" s="6"/>
       <c r="E114" s="7"/>
       <c r="F114" s="6"/>
@@ -3122,8 +3159,8 @@
       </c>
     </row>
     <row r="115" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B115" s="24"/>
-      <c r="C115" s="24"/>
+      <c r="B115" s="16"/>
+      <c r="C115" s="16"/>
       <c r="D115" s="10"/>
       <c r="E115" s="11"/>
       <c r="F115" s="10"/>
@@ -3140,15 +3177,15 @@
       </c>
     </row>
     <row r="116" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B116" s="24"/>
-      <c r="C116" s="24"/>
+      <c r="B116" s="16"/>
+      <c r="C116" s="16"/>
       <c r="D116" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E116" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="F116" s="16" t="s">
+      <c r="F116" s="18" t="s">
         <v>167</v>
       </c>
       <c r="G116" s="6" t="s">
@@ -3165,49 +3202,233 @@
       </c>
     </row>
     <row r="117" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B117" s="24"/>
-      <c r="C117" s="24"/>
-      <c r="D117" s="10"/>
-      <c r="E117" s="11"/>
+      <c r="B117" s="26"/>
+      <c r="C117" s="26"/>
+      <c r="D117" s="6"/>
+      <c r="E117" s="7"/>
       <c r="F117" s="18"/>
-      <c r="G117" s="10"/>
-      <c r="H117" s="10"/>
-      <c r="I117" s="10" t="s">
+      <c r="G117" s="6"/>
+      <c r="H117" s="6"/>
+      <c r="I117" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="J117" s="10" t="s">
+      <c r="J117" s="6" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="118" spans="2:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="118" spans="2:11" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B118" s="26" t="s">
+        <v>173</v>
+      </c>
+      <c r="C118" s="26" t="s">
+        <v>122</v>
+      </c>
+      <c r="D118" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E118" s="23" t="s">
+        <v>176</v>
+      </c>
+      <c r="F118" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G118" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="H118" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I118" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="J118" s="31" t="s">
+        <v>79</v>
+      </c>
+      <c r="K118" s="30" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="119" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B119" s="17"/>
+      <c r="C119" s="17"/>
+      <c r="D119" s="6"/>
+      <c r="E119" s="20"/>
+      <c r="F119" s="6"/>
+      <c r="G119" s="6"/>
+      <c r="H119" s="6"/>
+      <c r="I119" s="6"/>
+      <c r="J119" s="6"/>
+    </row>
+    <row r="120" spans="2:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B120" s="17"/>
+      <c r="C120" s="17"/>
+      <c r="D120" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E120" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="F120" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G120" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="H120" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I120" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="J120" s="31" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="121" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B121" s="17"/>
+      <c r="C121" s="17"/>
+      <c r="D121" s="10"/>
+      <c r="E121" s="15"/>
+      <c r="F121" s="10"/>
+      <c r="G121" s="10"/>
+      <c r="H121" s="10"/>
+      <c r="I121" s="32" t="s">
+        <v>28</v>
+      </c>
+      <c r="J121" s="10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="122" spans="2:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B122" s="17"/>
+      <c r="C122" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="D122" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E122" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="F122" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="G122" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="H122" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="I122" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="J122" s="29" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="123" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B123" s="17"/>
+      <c r="C123" s="17"/>
+      <c r="D123" s="6"/>
+      <c r="E123" s="7"/>
+      <c r="F123" s="6"/>
+      <c r="G123" s="6"/>
+      <c r="H123" s="6"/>
+      <c r="I123" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="J123" s="29" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="124" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B124" s="17"/>
+      <c r="C124" s="17"/>
+      <c r="D124" s="6"/>
+      <c r="E124" s="7"/>
+      <c r="F124" s="6"/>
+      <c r="G124" s="6"/>
+      <c r="H124" s="6"/>
+      <c r="I124" s="6"/>
+      <c r="J124" s="6"/>
+    </row>
+    <row r="125" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B125" s="17"/>
+      <c r="C125" s="17"/>
+      <c r="D125" s="6"/>
+      <c r="E125" s="7"/>
+      <c r="F125" s="6"/>
+      <c r="G125" s="6"/>
+      <c r="H125" s="6"/>
+      <c r="I125" s="6"/>
+      <c r="J125" s="6"/>
+    </row>
+    <row r="126" spans="2:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B126" s="17"/>
+      <c r="C126" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="D126" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E126" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="F126" s="21" t="s">
+        <v>182</v>
+      </c>
+      <c r="G126" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="H126" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I126" s="31" t="s">
+        <v>14</v>
+      </c>
+      <c r="J126" s="31" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="127" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B127" s="17"/>
+      <c r="C127" s="18"/>
+      <c r="D127" s="6"/>
+      <c r="E127" s="7"/>
+      <c r="F127" s="18"/>
+      <c r="G127" s="6"/>
+      <c r="H127" s="6"/>
+      <c r="I127" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="J127" s="29" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="128" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B128" s="27"/>
+      <c r="C128" s="19"/>
+      <c r="D128" s="10"/>
+      <c r="E128" s="11"/>
+      <c r="F128" s="10"/>
+      <c r="G128" s="10"/>
+      <c r="H128" s="10"/>
+      <c r="I128" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="J128" s="10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="129" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="40">
-    <mergeCell ref="C106:C117"/>
-    <mergeCell ref="B101:B117"/>
-    <mergeCell ref="F106:F108"/>
-    <mergeCell ref="F116:F117"/>
-    <mergeCell ref="B93:B100"/>
-    <mergeCell ref="E95:E97"/>
-    <mergeCell ref="C101:C105"/>
-    <mergeCell ref="G84:G85"/>
-    <mergeCell ref="C82:C92"/>
-    <mergeCell ref="B82:B92"/>
-    <mergeCell ref="G95:G96"/>
-    <mergeCell ref="G103:G104"/>
-    <mergeCell ref="F82:F83"/>
-    <mergeCell ref="F71:F73"/>
-    <mergeCell ref="E77:E79"/>
-    <mergeCell ref="E80:E81"/>
-    <mergeCell ref="C93:C100"/>
-    <mergeCell ref="G56:G57"/>
-    <mergeCell ref="C38:C55"/>
-    <mergeCell ref="C56:C70"/>
-    <mergeCell ref="C77:C81"/>
-    <mergeCell ref="B71:B81"/>
-    <mergeCell ref="F74:F76"/>
-    <mergeCell ref="C71:C76"/>
-    <mergeCell ref="G77:G79"/>
-    <mergeCell ref="G80:G81"/>
+  <mergeCells count="46">
+    <mergeCell ref="B118:B128"/>
+    <mergeCell ref="E118:E119"/>
+    <mergeCell ref="F126:F127"/>
+    <mergeCell ref="C118:C121"/>
+    <mergeCell ref="C122:C125"/>
+    <mergeCell ref="C126:C128"/>
     <mergeCell ref="B22:B37"/>
     <mergeCell ref="E63:E64"/>
     <mergeCell ref="G11:G13"/>
@@ -3222,6 +3443,32 @@
     <mergeCell ref="C35:C37"/>
     <mergeCell ref="B38:B70"/>
     <mergeCell ref="F56:F57"/>
+    <mergeCell ref="C38:C55"/>
+    <mergeCell ref="C56:C70"/>
+    <mergeCell ref="C77:C81"/>
+    <mergeCell ref="B71:B81"/>
+    <mergeCell ref="F74:F76"/>
+    <mergeCell ref="C71:C76"/>
+    <mergeCell ref="F71:F73"/>
+    <mergeCell ref="E77:E79"/>
+    <mergeCell ref="E80:E81"/>
+    <mergeCell ref="C93:C100"/>
+    <mergeCell ref="G56:G57"/>
+    <mergeCell ref="G77:G79"/>
+    <mergeCell ref="G80:G81"/>
+    <mergeCell ref="G84:G85"/>
+    <mergeCell ref="C82:C92"/>
+    <mergeCell ref="B82:B92"/>
+    <mergeCell ref="G95:G96"/>
+    <mergeCell ref="G103:G104"/>
+    <mergeCell ref="F82:F83"/>
+    <mergeCell ref="C106:C117"/>
+    <mergeCell ref="B101:B117"/>
+    <mergeCell ref="F106:F108"/>
+    <mergeCell ref="F116:F117"/>
+    <mergeCell ref="B93:B100"/>
+    <mergeCell ref="E95:E97"/>
+    <mergeCell ref="C101:C105"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Feat(chore): Agrego diagrama de clases y modifico diagrama de estados
</commit_message>
<xml_diff>
--- a/docs/Diagramas_Actuales/Endpoints.xlsx
+++ b/docs/Diagramas_Actuales/Endpoints.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\agusp\OneDrive\Escritorio\UNLaM\Proyecto_Stock_Fullstack\docs\Diagramas_Actuales\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23E15A69-0EA1-4BEA-8BA8-3E8C298DE16F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DD107A14-4AF5-460B-A511-CE5486F3841C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00198741-A7AD-4B5A-8F84-9858E7D73BD8}"/>
   </bookViews>
@@ -720,16 +720,20 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -738,31 +742,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1123,10 +1123,10 @@
       </c>
     </row>
     <row r="11" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="29" t="s">
         <v>57</v>
       </c>
       <c r="D11" s="4" t="s">
@@ -1138,7 +1138,7 @@
       <c r="F11" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G11" s="21" t="s">
+      <c r="G11" s="25" t="s">
         <v>21</v>
       </c>
       <c r="H11" s="4" t="s">
@@ -1155,12 +1155,12 @@
       </c>
     </row>
     <row r="12" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
+      <c r="B12" s="29"/>
+      <c r="C12" s="29"/>
       <c r="D12" s="6"/>
       <c r="E12" s="7"/>
       <c r="F12" s="6"/>
-      <c r="G12" s="18"/>
+      <c r="G12" s="26"/>
       <c r="H12" s="6"/>
       <c r="I12" s="6" t="s">
         <v>17</v>
@@ -1173,12 +1173,12 @@
       </c>
     </row>
     <row r="13" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="29"/>
       <c r="D13" s="6"/>
       <c r="E13" s="7"/>
       <c r="F13" s="6"/>
-      <c r="G13" s="18"/>
+      <c r="G13" s="26"/>
       <c r="H13" s="6"/>
       <c r="I13" s="6" t="s">
         <v>19</v>
@@ -1191,8 +1191,8 @@
       </c>
     </row>
     <row r="14" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="16"/>
-      <c r="C14" s="16"/>
+      <c r="B14" s="29"/>
+      <c r="C14" s="29"/>
       <c r="D14" s="10"/>
       <c r="E14" s="11"/>
       <c r="F14" s="10"/>
@@ -1206,8 +1206,8 @@
       </c>
     </row>
     <row r="15" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="29"/>
       <c r="D15" s="4" t="s">
         <v>8</v>
       </c>
@@ -1217,7 +1217,7 @@
       <c r="F15" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="G15" s="26" t="s">
+      <c r="G15" s="20" t="s">
         <v>41</v>
       </c>
       <c r="H15" s="4" t="s">
@@ -1231,12 +1231,12 @@
       </c>
     </row>
     <row r="16" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="16"/>
-      <c r="C16" s="16"/>
+      <c r="B16" s="29"/>
+      <c r="C16" s="29"/>
       <c r="D16" s="6"/>
       <c r="E16" s="7"/>
       <c r="F16" s="6"/>
-      <c r="G16" s="17"/>
+      <c r="G16" s="21"/>
       <c r="H16" s="6" t="s">
         <v>38</v>
       </c>
@@ -1244,19 +1244,19 @@
       <c r="J16" s="6"/>
     </row>
     <row r="17" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="16"/>
-      <c r="C17" s="16"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="29"/>
       <c r="D17" s="10"/>
       <c r="E17" s="11"/>
       <c r="F17" s="10"/>
-      <c r="G17" s="27"/>
+      <c r="G17" s="22"/>
       <c r="H17" s="10"/>
       <c r="I17" s="10"/>
       <c r="J17" s="10"/>
     </row>
     <row r="18" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="16"/>
-      <c r="C18" s="16"/>
+      <c r="B18" s="29"/>
+      <c r="C18" s="29"/>
       <c r="D18" s="6" t="s">
         <v>8</v>
       </c>
@@ -1280,8 +1280,8 @@
       </c>
     </row>
     <row r="19" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="16"/>
-      <c r="C19" s="16"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
       <c r="D19" s="6"/>
       <c r="E19" s="7"/>
       <c r="F19" s="6"/>
@@ -1295,8 +1295,8 @@
       </c>
     </row>
     <row r="20" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="16"/>
-      <c r="C20" s="16"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
       <c r="D20" s="6"/>
       <c r="E20" s="7"/>
       <c r="F20" s="6"/>
@@ -1310,8 +1310,8 @@
       </c>
     </row>
     <row r="21" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="16"/>
-      <c r="C21" s="16"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
       <c r="D21" s="10"/>
       <c r="E21" s="11"/>
       <c r="F21" s="10"/>
@@ -1325,10 +1325,10 @@
       </c>
     </row>
     <row r="22" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="22" t="s">
+      <c r="B22" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="16" t="s">
+      <c r="C22" s="29" t="s">
         <v>58</v>
       </c>
       <c r="D22" s="4" t="s">
@@ -1337,7 +1337,7 @@
       <c r="E22" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="F22" s="21" t="s">
+      <c r="F22" s="25" t="s">
         <v>24</v>
       </c>
       <c r="G22" s="4" t="s">
@@ -1354,11 +1354,11 @@
       </c>
     </row>
     <row r="23" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="22"/>
-      <c r="C23" s="16"/>
+      <c r="B23" s="28"/>
+      <c r="C23" s="29"/>
       <c r="D23" s="6"/>
       <c r="E23" s="7"/>
-      <c r="F23" s="18"/>
+      <c r="F23" s="26"/>
       <c r="G23" s="6"/>
       <c r="H23" s="6"/>
       <c r="I23" s="6" t="s">
@@ -1372,19 +1372,19 @@
       </c>
     </row>
     <row r="24" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="22"/>
-      <c r="C24" s="16"/>
+      <c r="B24" s="28"/>
+      <c r="C24" s="29"/>
       <c r="D24" s="6"/>
       <c r="E24" s="7"/>
-      <c r="F24" s="18"/>
+      <c r="F24" s="26"/>
       <c r="G24" s="6"/>
       <c r="H24" s="6"/>
       <c r="I24" s="6"/>
       <c r="J24" s="6"/>
     </row>
     <row r="25" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="22"/>
-      <c r="C25" s="16"/>
+      <c r="B25" s="28"/>
+      <c r="C25" s="29"/>
       <c r="D25" s="10"/>
       <c r="E25" s="11"/>
       <c r="F25" s="10"/>
@@ -1398,15 +1398,15 @@
       </c>
     </row>
     <row r="26" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="22"/>
-      <c r="C26" s="16"/>
+      <c r="B26" s="28"/>
+      <c r="C26" s="29"/>
       <c r="D26" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="F26" s="18" t="s">
+      <c r="F26" s="26" t="s">
         <v>32</v>
       </c>
       <c r="G26" s="6" t="s">
@@ -1423,11 +1423,11 @@
       </c>
     </row>
     <row r="27" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="22"/>
-      <c r="C27" s="16"/>
+      <c r="B27" s="28"/>
+      <c r="C27" s="29"/>
       <c r="D27" s="6"/>
       <c r="E27" s="7"/>
-      <c r="F27" s="18"/>
+      <c r="F27" s="26"/>
       <c r="G27" s="6"/>
       <c r="H27" s="6"/>
       <c r="I27" s="6" t="s">
@@ -1441,19 +1441,19 @@
       </c>
     </row>
     <row r="28" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="22"/>
-      <c r="C28" s="16"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="29"/>
       <c r="D28" s="6"/>
       <c r="E28" s="7"/>
-      <c r="F28" s="18"/>
+      <c r="F28" s="26"/>
       <c r="G28" s="6"/>
       <c r="H28" s="6"/>
       <c r="I28" s="6"/>
       <c r="J28" s="6"/>
     </row>
     <row r="29" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="22"/>
-      <c r="C29" s="16"/>
+      <c r="B29" s="28"/>
+      <c r="C29" s="29"/>
       <c r="D29" s="6"/>
       <c r="E29" s="7"/>
       <c r="F29" s="6"/>
@@ -1467,8 +1467,8 @@
       </c>
     </row>
     <row r="30" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="22"/>
-      <c r="C30" s="16"/>
+      <c r="B30" s="28"/>
+      <c r="C30" s="29"/>
       <c r="D30" s="4" t="s">
         <v>9</v>
       </c>
@@ -1495,8 +1495,8 @@
       </c>
     </row>
     <row r="31" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="22"/>
-      <c r="C31" s="16"/>
+      <c r="B31" s="28"/>
+      <c r="C31" s="29"/>
       <c r="D31" s="6"/>
       <c r="E31" s="7"/>
       <c r="F31" s="6"/>
@@ -1513,8 +1513,8 @@
       </c>
     </row>
     <row r="32" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="22"/>
-      <c r="C32" s="16"/>
+      <c r="B32" s="28"/>
+      <c r="C32" s="29"/>
       <c r="D32" s="10"/>
       <c r="E32" s="11"/>
       <c r="F32" s="10"/>
@@ -1524,8 +1524,8 @@
       <c r="J32" s="10"/>
     </row>
     <row r="33" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="22"/>
-      <c r="C33" s="16"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="29"/>
       <c r="D33" s="6" t="s">
         <v>51</v>
       </c>
@@ -1535,7 +1535,7 @@
       <c r="F33" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="G33" s="18" t="s">
+      <c r="G33" s="26" t="s">
         <v>53</v>
       </c>
       <c r="H33" s="6" t="s">
@@ -1552,19 +1552,19 @@
       </c>
     </row>
     <row r="34" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="22"/>
-      <c r="C34" s="26"/>
+      <c r="B34" s="28"/>
+      <c r="C34" s="20"/>
       <c r="D34" s="6"/>
       <c r="E34" s="7"/>
       <c r="F34" s="6"/>
-      <c r="G34" s="18"/>
+      <c r="G34" s="26"/>
       <c r="H34" s="6"/>
       <c r="I34" s="6"/>
       <c r="J34" s="6"/>
     </row>
     <row r="35" spans="2:11" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="22"/>
-      <c r="C35" s="28" t="s">
+      <c r="B35" s="28"/>
+      <c r="C35" s="30" t="s">
         <v>88</v>
       </c>
       <c r="D35" s="4" t="s">
@@ -1576,7 +1576,7 @@
       <c r="F35" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="G35" s="21" t="s">
+      <c r="G35" s="25" t="s">
         <v>102</v>
       </c>
       <c r="H35" s="4" t="s">
@@ -1590,23 +1590,23 @@
       </c>
     </row>
     <row r="36" spans="2:11" ht="16.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="22"/>
-      <c r="C36" s="16"/>
+      <c r="B36" s="28"/>
+      <c r="C36" s="29"/>
       <c r="D36" s="6"/>
       <c r="E36" s="7"/>
       <c r="F36" s="6"/>
-      <c r="G36" s="18"/>
+      <c r="G36" s="26"/>
       <c r="H36" s="6"/>
       <c r="I36" s="6"/>
       <c r="J36" s="6"/>
     </row>
     <row r="37" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="22"/>
-      <c r="C37" s="16"/>
+      <c r="B37" s="28"/>
+      <c r="C37" s="29"/>
       <c r="D37" s="10"/>
       <c r="E37" s="11"/>
       <c r="F37" s="10"/>
-      <c r="G37" s="19"/>
+      <c r="G37" s="27"/>
       <c r="H37" s="10"/>
       <c r="I37" s="10"/>
       <c r="J37" s="10"/>
@@ -1615,10 +1615,10 @@
       </c>
     </row>
     <row r="38" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="16" t="s">
+      <c r="B38" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="C38" s="16" t="s">
+      <c r="C38" s="29" t="s">
         <v>59</v>
       </c>
       <c r="D38" s="6" t="s">
@@ -1647,8 +1647,8 @@
       </c>
     </row>
     <row r="39" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="16"/>
-      <c r="C39" s="16"/>
+      <c r="B39" s="29"/>
+      <c r="C39" s="29"/>
       <c r="D39" s="6"/>
       <c r="E39" s="7"/>
       <c r="F39" s="6"/>
@@ -1662,8 +1662,8 @@
       </c>
     </row>
     <row r="40" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="16"/>
-      <c r="C40" s="16"/>
+      <c r="B40" s="29"/>
+      <c r="C40" s="29"/>
       <c r="D40" s="6"/>
       <c r="E40" s="7"/>
       <c r="F40" s="6"/>
@@ -1677,8 +1677,8 @@
       </c>
     </row>
     <row r="41" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="16"/>
-      <c r="C41" s="16"/>
+      <c r="B41" s="29"/>
+      <c r="C41" s="29"/>
       <c r="D41" s="6"/>
       <c r="E41" s="7"/>
       <c r="F41" s="6"/>
@@ -1695,8 +1695,8 @@
       </c>
     </row>
     <row r="42" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="16"/>
-      <c r="C42" s="16"/>
+      <c r="B42" s="29"/>
+      <c r="C42" s="29"/>
       <c r="D42" s="6"/>
       <c r="E42" s="7"/>
       <c r="F42" s="6"/>
@@ -1713,8 +1713,8 @@
       </c>
     </row>
     <row r="43" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="16"/>
-      <c r="C43" s="16"/>
+      <c r="B43" s="29"/>
+      <c r="C43" s="29"/>
       <c r="D43" s="4" t="s">
         <v>9</v>
       </c>
@@ -1738,8 +1738,8 @@
       </c>
     </row>
     <row r="44" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="16"/>
-      <c r="C44" s="16"/>
+      <c r="B44" s="29"/>
+      <c r="C44" s="29"/>
       <c r="D44" s="6"/>
       <c r="E44" s="7" t="s">
         <v>104</v>
@@ -1755,8 +1755,8 @@
       </c>
     </row>
     <row r="45" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="16"/>
-      <c r="C45" s="16"/>
+      <c r="B45" s="29"/>
+      <c r="C45" s="29"/>
       <c r="D45" s="10"/>
       <c r="E45" s="11"/>
       <c r="F45" s="10"/>
@@ -1773,8 +1773,8 @@
       </c>
     </row>
     <row r="46" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="16"/>
-      <c r="C46" s="16"/>
+      <c r="B46" s="29"/>
+      <c r="C46" s="29"/>
       <c r="D46" s="6" t="s">
         <v>9</v>
       </c>
@@ -1798,8 +1798,8 @@
       </c>
     </row>
     <row r="47" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="16"/>
-      <c r="C47" s="16"/>
+      <c r="B47" s="29"/>
+      <c r="C47" s="29"/>
       <c r="D47" s="6"/>
       <c r="E47" s="7" t="s">
         <v>105</v>
@@ -1815,8 +1815,8 @@
       </c>
     </row>
     <row r="48" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B48" s="16"/>
-      <c r="C48" s="16"/>
+      <c r="B48" s="29"/>
+      <c r="C48" s="29"/>
       <c r="D48" s="6"/>
       <c r="E48" s="7"/>
       <c r="F48" s="6"/>
@@ -1833,8 +1833,8 @@
       </c>
     </row>
     <row r="49" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="16"/>
-      <c r="C49" s="16"/>
+      <c r="B49" s="29"/>
+      <c r="C49" s="29"/>
       <c r="D49" s="4" t="s">
         <v>9</v>
       </c>
@@ -1858,8 +1858,8 @@
       </c>
     </row>
     <row r="50" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B50" s="16"/>
-      <c r="C50" s="16"/>
+      <c r="B50" s="29"/>
+      <c r="C50" s="29"/>
       <c r="D50" s="6"/>
       <c r="E50" s="7" t="s">
         <v>106</v>
@@ -1875,8 +1875,8 @@
       </c>
     </row>
     <row r="51" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B51" s="16"/>
-      <c r="C51" s="16"/>
+      <c r="B51" s="29"/>
+      <c r="C51" s="29"/>
       <c r="D51" s="10"/>
       <c r="E51" s="11"/>
       <c r="F51" s="10"/>
@@ -1893,8 +1893,8 @@
       </c>
     </row>
     <row r="52" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="16"/>
-      <c r="C52" s="16"/>
+      <c r="B52" s="29"/>
+      <c r="C52" s="29"/>
       <c r="D52" s="6" t="s">
         <v>8</v>
       </c>
@@ -1918,8 +1918,8 @@
       </c>
     </row>
     <row r="53" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B53" s="16"/>
-      <c r="C53" s="16"/>
+      <c r="B53" s="29"/>
+      <c r="C53" s="29"/>
       <c r="D53" s="6"/>
       <c r="E53" s="7"/>
       <c r="F53" s="6"/>
@@ -1933,8 +1933,8 @@
       </c>
     </row>
     <row r="54" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B54" s="16"/>
-      <c r="C54" s="16"/>
+      <c r="B54" s="29"/>
+      <c r="C54" s="29"/>
       <c r="D54" s="6"/>
       <c r="E54" s="7"/>
       <c r="F54" s="6"/>
@@ -1951,8 +1951,8 @@
       </c>
     </row>
     <row r="55" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="16"/>
-      <c r="C55" s="16"/>
+      <c r="B55" s="29"/>
+      <c r="C55" s="29"/>
       <c r="D55" s="6"/>
       <c r="E55" s="7"/>
       <c r="F55" s="6"/>
@@ -1969,8 +1969,8 @@
       </c>
     </row>
     <row r="56" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="16"/>
-      <c r="C56" s="16" t="s">
+      <c r="B56" s="29"/>
+      <c r="C56" s="29" t="s">
         <v>88</v>
       </c>
       <c r="D56" s="4" t="s">
@@ -1979,10 +1979,10 @@
       <c r="E56" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="F56" s="21" t="s">
+      <c r="F56" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="G56" s="21" t="s">
+      <c r="G56" s="25" t="s">
         <v>92</v>
       </c>
       <c r="H56" s="4" t="s">
@@ -1999,12 +1999,12 @@
       </c>
     </row>
     <row r="57" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B57" s="16"/>
-      <c r="C57" s="16"/>
+      <c r="B57" s="29"/>
+      <c r="C57" s="29"/>
       <c r="D57" s="6"/>
       <c r="E57" s="7"/>
-      <c r="F57" s="18"/>
-      <c r="G57" s="18"/>
+      <c r="F57" s="26"/>
+      <c r="G57" s="26"/>
       <c r="H57" s="6"/>
       <c r="I57" s="6" t="s">
         <v>19</v>
@@ -2017,8 +2017,8 @@
       </c>
     </row>
     <row r="58" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B58" s="16"/>
-      <c r="C58" s="16"/>
+      <c r="B58" s="29"/>
+      <c r="C58" s="29"/>
       <c r="D58" s="10"/>
       <c r="E58" s="11"/>
       <c r="F58" s="10"/>
@@ -2035,8 +2035,8 @@
       </c>
     </row>
     <row r="59" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="16"/>
-      <c r="C59" s="16"/>
+      <c r="B59" s="29"/>
+      <c r="C59" s="29"/>
       <c r="D59" s="6" t="s">
         <v>51</v>
       </c>
@@ -2060,8 +2060,8 @@
       </c>
     </row>
     <row r="60" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="16"/>
-      <c r="C60" s="16"/>
+      <c r="B60" s="29"/>
+      <c r="C60" s="29"/>
       <c r="D60" s="6"/>
       <c r="E60" s="7"/>
       <c r="F60" s="6"/>
@@ -2078,8 +2078,8 @@
       </c>
     </row>
     <row r="61" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="16"/>
-      <c r="C61" s="16"/>
+      <c r="B61" s="29"/>
+      <c r="C61" s="29"/>
       <c r="D61" s="4" t="s">
         <v>51</v>
       </c>
@@ -2103,8 +2103,8 @@
       </c>
     </row>
     <row r="62" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B62" s="16"/>
-      <c r="C62" s="16"/>
+      <c r="B62" s="29"/>
+      <c r="C62" s="29"/>
       <c r="D62" s="10"/>
       <c r="E62" s="11"/>
       <c r="F62" s="10"/>
@@ -2118,12 +2118,12 @@
       </c>
     </row>
     <row r="63" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B63" s="16"/>
-      <c r="C63" s="16"/>
+      <c r="B63" s="29"/>
+      <c r="C63" s="29"/>
       <c r="D63" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E63" s="20" t="s">
+      <c r="E63" s="24" t="s">
         <v>68</v>
       </c>
       <c r="F63" s="6" t="s">
@@ -2143,10 +2143,10 @@
       </c>
     </row>
     <row r="64" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="16"/>
-      <c r="C64" s="16"/>
+      <c r="B64" s="29"/>
+      <c r="C64" s="29"/>
       <c r="D64" s="6"/>
-      <c r="E64" s="20"/>
+      <c r="E64" s="24"/>
       <c r="F64" s="6"/>
       <c r="G64" s="6"/>
       <c r="H64" s="6"/>
@@ -2158,8 +2158,8 @@
       </c>
     </row>
     <row r="65" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B65" s="16"/>
-      <c r="C65" s="16"/>
+      <c r="B65" s="29"/>
+      <c r="C65" s="29"/>
       <c r="D65" s="2" t="s">
         <v>51</v>
       </c>
@@ -2183,8 +2183,8 @@
       </c>
     </row>
     <row r="66" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B66" s="16"/>
-      <c r="C66" s="16"/>
+      <c r="B66" s="29"/>
+      <c r="C66" s="29"/>
       <c r="D66" s="6" t="s">
         <v>9</v>
       </c>
@@ -2207,8 +2207,8 @@
       </c>
     </row>
     <row r="67" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B67" s="16"/>
-      <c r="C67" s="16"/>
+      <c r="B67" s="29"/>
+      <c r="C67" s="29"/>
       <c r="D67" s="6"/>
       <c r="E67" s="7"/>
       <c r="F67" s="6"/>
@@ -2225,8 +2225,8 @@
       </c>
     </row>
     <row r="68" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B68" s="16"/>
-      <c r="C68" s="16"/>
+      <c r="B68" s="29"/>
+      <c r="C68" s="29"/>
       <c r="D68" s="6"/>
       <c r="E68" s="7"/>
       <c r="F68" s="6"/>
@@ -2240,8 +2240,8 @@
       </c>
     </row>
     <row r="69" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B69" s="16"/>
-      <c r="C69" s="16"/>
+      <c r="B69" s="29"/>
+      <c r="C69" s="29"/>
       <c r="D69" s="4" t="s">
         <v>9</v>
       </c>
@@ -2268,8 +2268,8 @@
       </c>
     </row>
     <row r="70" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B70" s="16"/>
-      <c r="C70" s="16"/>
+      <c r="B70" s="29"/>
+      <c r="C70" s="29"/>
       <c r="D70" s="10"/>
       <c r="E70" s="11" t="s">
         <v>106</v>
@@ -2285,10 +2285,10 @@
       </c>
     </row>
     <row r="71" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B71" s="16" t="s">
+      <c r="B71" s="29" t="s">
         <v>110</v>
       </c>
-      <c r="C71" s="16" t="s">
+      <c r="C71" s="29" t="s">
         <v>121</v>
       </c>
       <c r="D71" s="6" t="s">
@@ -2297,7 +2297,7 @@
       <c r="E71" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="F71" s="18" t="s">
+      <c r="F71" s="26" t="s">
         <v>115</v>
       </c>
       <c r="G71" s="6" t="s">
@@ -2317,11 +2317,11 @@
       </c>
     </row>
     <row r="72" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B72" s="16"/>
-      <c r="C72" s="16"/>
+      <c r="B72" s="29"/>
+      <c r="C72" s="29"/>
       <c r="D72" s="6"/>
       <c r="E72" s="7"/>
-      <c r="F72" s="18"/>
+      <c r="F72" s="26"/>
       <c r="G72" s="6"/>
       <c r="H72" s="6"/>
       <c r="I72" s="6" t="s">
@@ -2335,11 +2335,11 @@
       </c>
     </row>
     <row r="73" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B73" s="16"/>
-      <c r="C73" s="16"/>
+      <c r="B73" s="29"/>
+      <c r="C73" s="29"/>
       <c r="D73" s="6"/>
       <c r="E73" s="7"/>
-      <c r="F73" s="18"/>
+      <c r="F73" s="26"/>
       <c r="G73" s="6"/>
       <c r="H73" s="6"/>
       <c r="I73" s="6" t="s">
@@ -2353,15 +2353,15 @@
       </c>
     </row>
     <row r="74" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B74" s="16"/>
-      <c r="C74" s="16"/>
+      <c r="B74" s="29"/>
+      <c r="C74" s="29"/>
       <c r="D74" s="4" t="s">
         <v>9</v>
       </c>
       <c r="E74" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="F74" s="21" t="s">
+      <c r="F74" s="25" t="s">
         <v>124</v>
       </c>
       <c r="G74" s="4" t="s">
@@ -2378,11 +2378,11 @@
       </c>
     </row>
     <row r="75" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B75" s="16"/>
-      <c r="C75" s="16"/>
+      <c r="B75" s="29"/>
+      <c r="C75" s="29"/>
       <c r="D75" s="6"/>
       <c r="E75" s="7"/>
-      <c r="F75" s="18"/>
+      <c r="F75" s="26"/>
       <c r="G75" s="6"/>
       <c r="H75" s="6"/>
       <c r="I75" s="6" t="s">
@@ -2393,11 +2393,11 @@
       </c>
     </row>
     <row r="76" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B76" s="16"/>
-      <c r="C76" s="16"/>
+      <c r="B76" s="29"/>
+      <c r="C76" s="29"/>
       <c r="D76" s="10"/>
       <c r="E76" s="11"/>
-      <c r="F76" s="19"/>
+      <c r="F76" s="27"/>
       <c r="G76" s="10"/>
       <c r="H76" s="10"/>
       <c r="I76" s="10" t="s">
@@ -2408,20 +2408,20 @@
       </c>
     </row>
     <row r="77" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B77" s="16"/>
-      <c r="C77" s="25" t="s">
+      <c r="B77" s="29"/>
+      <c r="C77" s="31" t="s">
         <v>122</v>
       </c>
       <c r="D77" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E77" s="20" t="s">
+      <c r="E77" s="24" t="s">
         <v>172</v>
       </c>
       <c r="F77" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="G77" s="18" t="s">
+      <c r="G77" s="26" t="s">
         <v>119</v>
       </c>
       <c r="H77" s="6" t="s">
@@ -2438,30 +2438,30 @@
       </c>
     </row>
     <row r="78" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B78" s="16"/>
-      <c r="C78" s="25"/>
+      <c r="B78" s="29"/>
+      <c r="C78" s="31"/>
       <c r="D78" s="6"/>
-      <c r="E78" s="20"/>
+      <c r="E78" s="24"/>
       <c r="F78" s="6"/>
-      <c r="G78" s="18"/>
+      <c r="G78" s="26"/>
       <c r="H78" s="6"/>
       <c r="I78" s="6"/>
       <c r="J78" s="6"/>
     </row>
     <row r="79" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B79" s="16"/>
-      <c r="C79" s="25"/>
+      <c r="B79" s="29"/>
+      <c r="C79" s="31"/>
       <c r="D79" s="6"/>
-      <c r="E79" s="20"/>
+      <c r="E79" s="24"/>
       <c r="F79" s="6"/>
-      <c r="G79" s="18"/>
+      <c r="G79" s="26"/>
       <c r="H79" s="6"/>
       <c r="I79" s="6"/>
       <c r="J79" s="6"/>
     </row>
     <row r="80" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B80" s="16"/>
-      <c r="C80" s="25"/>
+      <c r="B80" s="29"/>
+      <c r="C80" s="31"/>
       <c r="D80" s="4" t="s">
         <v>51</v>
       </c>
@@ -2471,7 +2471,7 @@
       <c r="F80" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="G80" s="21" t="s">
+      <c r="G80" s="25" t="s">
         <v>120</v>
       </c>
       <c r="H80" s="4" t="s">
@@ -2485,21 +2485,21 @@
       </c>
     </row>
     <row r="81" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B81" s="16"/>
-      <c r="C81" s="25"/>
+      <c r="B81" s="29"/>
+      <c r="C81" s="31"/>
       <c r="D81" s="10"/>
-      <c r="E81" s="24"/>
+      <c r="E81" s="32"/>
       <c r="F81" s="10"/>
-      <c r="G81" s="19"/>
+      <c r="G81" s="27"/>
       <c r="H81" s="10"/>
       <c r="I81" s="10"/>
       <c r="J81" s="10"/>
     </row>
     <row r="82" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B82" s="22" t="s">
+      <c r="B82" s="28" t="s">
         <v>137</v>
       </c>
-      <c r="C82" s="16" t="s">
+      <c r="C82" s="29" t="s">
         <v>88</v>
       </c>
       <c r="D82" s="6" t="s">
@@ -2508,7 +2508,7 @@
       <c r="E82" s="7" t="s">
         <v>126</v>
       </c>
-      <c r="F82" s="18" t="s">
+      <c r="F82" s="26" t="s">
         <v>127</v>
       </c>
       <c r="G82" s="6" t="s">
@@ -2528,11 +2528,11 @@
       </c>
     </row>
     <row r="83" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B83" s="22"/>
-      <c r="C83" s="16"/>
+      <c r="B83" s="28"/>
+      <c r="C83" s="29"/>
       <c r="D83" s="6"/>
       <c r="E83" s="7"/>
-      <c r="F83" s="18"/>
+      <c r="F83" s="26"/>
       <c r="G83" s="6"/>
       <c r="H83" s="6"/>
       <c r="I83" s="6" t="s">
@@ -2543,8 +2543,8 @@
       </c>
     </row>
     <row r="84" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B84" s="22"/>
-      <c r="C84" s="16"/>
+      <c r="B84" s="28"/>
+      <c r="C84" s="29"/>
       <c r="D84" s="4" t="s">
         <v>51</v>
       </c>
@@ -2554,7 +2554,7 @@
       <c r="F84" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="G84" s="21" t="s">
+      <c r="G84" s="25" t="s">
         <v>130</v>
       </c>
       <c r="H84" s="4" t="s">
@@ -2571,21 +2571,21 @@
       </c>
     </row>
     <row r="85" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B85" s="22"/>
-      <c r="C85" s="16"/>
+      <c r="B85" s="28"/>
+      <c r="C85" s="29"/>
       <c r="D85" s="10"/>
       <c r="E85" s="11" t="s">
         <v>132</v>
       </c>
       <c r="F85" s="13"/>
-      <c r="G85" s="19"/>
+      <c r="G85" s="27"/>
       <c r="H85" s="10"/>
       <c r="I85" s="10"/>
       <c r="J85" s="10"/>
     </row>
     <row r="86" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B86" s="22"/>
-      <c r="C86" s="16"/>
+      <c r="B86" s="28"/>
+      <c r="C86" s="29"/>
       <c r="D86" s="6" t="s">
         <v>51</v>
       </c>
@@ -2609,8 +2609,8 @@
       </c>
     </row>
     <row r="87" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B87" s="22"/>
-      <c r="C87" s="16"/>
+      <c r="B87" s="28"/>
+      <c r="C87" s="29"/>
       <c r="D87" s="6"/>
       <c r="E87" s="7"/>
       <c r="F87" s="6"/>
@@ -2624,8 +2624,8 @@
       </c>
     </row>
     <row r="88" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B88" s="22"/>
-      <c r="C88" s="16"/>
+      <c r="B88" s="28"/>
+      <c r="C88" s="29"/>
       <c r="D88" s="4" t="s">
         <v>9</v>
       </c>
@@ -2652,8 +2652,8 @@
       </c>
     </row>
     <row r="89" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B89" s="22"/>
-      <c r="C89" s="16"/>
+      <c r="B89" s="28"/>
+      <c r="C89" s="29"/>
       <c r="D89" s="10"/>
       <c r="E89" s="11"/>
       <c r="F89" s="10"/>
@@ -2667,8 +2667,8 @@
       </c>
     </row>
     <row r="90" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B90" s="22"/>
-      <c r="C90" s="16"/>
+      <c r="B90" s="28"/>
+      <c r="C90" s="29"/>
       <c r="D90" s="6" t="s">
         <v>9</v>
       </c>
@@ -2695,8 +2695,8 @@
       </c>
     </row>
     <row r="91" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B91" s="22"/>
-      <c r="C91" s="16"/>
+      <c r="B91" s="28"/>
+      <c r="C91" s="29"/>
       <c r="D91" s="6"/>
       <c r="E91" s="7"/>
       <c r="F91" s="6"/>
@@ -2710,8 +2710,8 @@
       </c>
     </row>
     <row r="92" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B92" s="22"/>
-      <c r="C92" s="16"/>
+      <c r="B92" s="28"/>
+      <c r="C92" s="29"/>
       <c r="D92" s="6"/>
       <c r="E92" s="7"/>
       <c r="F92" s="6"/>
@@ -2725,10 +2725,10 @@
       </c>
     </row>
     <row r="93" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B93" s="16" t="s">
+      <c r="B93" s="29" t="s">
         <v>109</v>
       </c>
-      <c r="C93" s="16" t="s">
+      <c r="C93" s="29" t="s">
         <v>122</v>
       </c>
       <c r="D93" s="4" t="s">
@@ -2754,8 +2754,8 @@
       </c>
     </row>
     <row r="94" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B94" s="16"/>
-      <c r="C94" s="16"/>
+      <c r="B94" s="29"/>
+      <c r="C94" s="29"/>
       <c r="D94" s="10"/>
       <c r="E94" s="11"/>
       <c r="F94" s="10"/>
@@ -2769,18 +2769,18 @@
       </c>
     </row>
     <row r="95" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B95" s="16"/>
-      <c r="C95" s="16"/>
+      <c r="B95" s="29"/>
+      <c r="C95" s="29"/>
       <c r="D95" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E95" s="20" t="s">
+      <c r="E95" s="24" t="s">
         <v>151</v>
       </c>
       <c r="F95" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="G95" s="18" t="s">
+      <c r="G95" s="26" t="s">
         <v>150</v>
       </c>
       <c r="H95" s="6" t="s">
@@ -2797,12 +2797,12 @@
       </c>
     </row>
     <row r="96" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B96" s="16"/>
-      <c r="C96" s="16"/>
+      <c r="B96" s="29"/>
+      <c r="C96" s="29"/>
       <c r="D96" s="6"/>
-      <c r="E96" s="20"/>
+      <c r="E96" s="24"/>
       <c r="F96" s="6"/>
-      <c r="G96" s="18"/>
+      <c r="G96" s="26"/>
       <c r="H96" s="6"/>
       <c r="I96" s="6" t="s">
         <v>19</v>
@@ -2812,10 +2812,10 @@
       </c>
     </row>
     <row r="97" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B97" s="16"/>
-      <c r="C97" s="16"/>
+      <c r="B97" s="29"/>
+      <c r="C97" s="29"/>
       <c r="D97" s="6"/>
-      <c r="E97" s="20"/>
+      <c r="E97" s="24"/>
       <c r="F97" s="6"/>
       <c r="G97" s="8"/>
       <c r="H97" s="6"/>
@@ -2826,8 +2826,8 @@
       </c>
     </row>
     <row r="98" spans="2:11" ht="15" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B98" s="16"/>
-      <c r="C98" s="16"/>
+      <c r="B98" s="29"/>
+      <c r="C98" s="29"/>
       <c r="D98" s="4" t="s">
         <v>51</v>
       </c>
@@ -2851,8 +2851,8 @@
       </c>
     </row>
     <row r="99" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B99" s="16"/>
-      <c r="C99" s="16"/>
+      <c r="B99" s="29"/>
+      <c r="C99" s="29"/>
       <c r="D99" s="6"/>
       <c r="E99" s="9"/>
       <c r="F99" s="6"/>
@@ -2866,8 +2866,8 @@
       </c>
     </row>
     <row r="100" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B100" s="16"/>
-      <c r="C100" s="16"/>
+      <c r="B100" s="29"/>
+      <c r="C100" s="29"/>
       <c r="D100" s="10"/>
       <c r="E100" s="15"/>
       <c r="F100" s="10"/>
@@ -2884,10 +2884,10 @@
       </c>
     </row>
     <row r="101" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B101" s="16" t="s">
+      <c r="B101" s="29" t="s">
         <v>153</v>
       </c>
-      <c r="C101" s="16" t="s">
+      <c r="C101" s="29" t="s">
         <v>154</v>
       </c>
       <c r="D101" s="6" t="s">
@@ -2913,8 +2913,8 @@
       </c>
     </row>
     <row r="102" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B102" s="16"/>
-      <c r="C102" s="16"/>
+      <c r="B102" s="29"/>
+      <c r="C102" s="29"/>
       <c r="D102" s="6"/>
       <c r="E102" s="7"/>
       <c r="F102" s="6"/>
@@ -2928,8 +2928,8 @@
       </c>
     </row>
     <row r="103" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B103" s="16"/>
-      <c r="C103" s="16"/>
+      <c r="B103" s="29"/>
+      <c r="C103" s="29"/>
       <c r="D103" s="4" t="s">
         <v>51</v>
       </c>
@@ -2939,7 +2939,7 @@
       <c r="F103" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="G103" s="21" t="s">
+      <c r="G103" s="25" t="s">
         <v>158</v>
       </c>
       <c r="H103" s="4" t="s">
@@ -2953,12 +2953,12 @@
       </c>
     </row>
     <row r="104" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B104" s="16"/>
-      <c r="C104" s="16"/>
+      <c r="B104" s="29"/>
+      <c r="C104" s="29"/>
       <c r="D104" s="6"/>
       <c r="E104" s="7"/>
       <c r="F104" s="6"/>
-      <c r="G104" s="18"/>
+      <c r="G104" s="26"/>
       <c r="H104" s="6"/>
       <c r="I104" s="6" t="s">
         <v>19</v>
@@ -2968,8 +2968,8 @@
       </c>
     </row>
     <row r="105" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B105" s="16"/>
-      <c r="C105" s="16"/>
+      <c r="B105" s="29"/>
+      <c r="C105" s="29"/>
       <c r="D105" s="10"/>
       <c r="E105" s="11"/>
       <c r="F105" s="10"/>
@@ -2983,8 +2983,8 @@
       </c>
     </row>
     <row r="106" spans="2:11" ht="30" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B106" s="16"/>
-      <c r="C106" s="16" t="s">
+      <c r="B106" s="29"/>
+      <c r="C106" s="29" t="s">
         <v>59</v>
       </c>
       <c r="D106" s="6" t="s">
@@ -2993,7 +2993,7 @@
       <c r="E106" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="F106" s="17" t="s">
+      <c r="F106" s="21" t="s">
         <v>170</v>
       </c>
       <c r="G106" s="6" t="s">
@@ -3010,11 +3010,11 @@
       </c>
     </row>
     <row r="107" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B107" s="16"/>
-      <c r="C107" s="16"/>
+      <c r="B107" s="29"/>
+      <c r="C107" s="29"/>
       <c r="D107" s="6"/>
       <c r="E107" s="7"/>
-      <c r="F107" s="17"/>
+      <c r="F107" s="21"/>
       <c r="G107" s="6"/>
       <c r="H107" s="6"/>
       <c r="I107" s="6" t="s">
@@ -3025,11 +3025,11 @@
       </c>
     </row>
     <row r="108" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B108" s="16"/>
-      <c r="C108" s="16"/>
+      <c r="B108" s="29"/>
+      <c r="C108" s="29"/>
       <c r="D108" s="6"/>
       <c r="E108" s="7"/>
-      <c r="F108" s="17"/>
+      <c r="F108" s="21"/>
       <c r="G108" s="6"/>
       <c r="H108" s="6"/>
       <c r="I108" s="6" t="s">
@@ -3043,8 +3043,8 @@
       </c>
     </row>
     <row r="109" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B109" s="16"/>
-      <c r="C109" s="16"/>
+      <c r="B109" s="29"/>
+      <c r="C109" s="29"/>
       <c r="D109" s="4" t="s">
         <v>85</v>
       </c>
@@ -3068,8 +3068,8 @@
       </c>
     </row>
     <row r="110" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B110" s="16"/>
-      <c r="C110" s="16"/>
+      <c r="B110" s="29"/>
+      <c r="C110" s="29"/>
       <c r="D110" s="6"/>
       <c r="E110" s="7"/>
       <c r="F110" s="6"/>
@@ -3083,8 +3083,8 @@
       </c>
     </row>
     <row r="111" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B111" s="16"/>
-      <c r="C111" s="16"/>
+      <c r="B111" s="29"/>
+      <c r="C111" s="29"/>
       <c r="D111" s="10"/>
       <c r="E111" s="11"/>
       <c r="F111" s="10"/>
@@ -3101,8 +3101,8 @@
       </c>
     </row>
     <row r="112" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B112" s="16"/>
-      <c r="C112" s="16"/>
+      <c r="B112" s="29"/>
+      <c r="C112" s="29"/>
       <c r="D112" s="4" t="s">
         <v>9</v>
       </c>
@@ -3129,8 +3129,8 @@
       </c>
     </row>
     <row r="113" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B113" s="16"/>
-      <c r="C113" s="16"/>
+      <c r="B113" s="29"/>
+      <c r="C113" s="29"/>
       <c r="D113" s="6"/>
       <c r="E113" s="7"/>
       <c r="F113" s="6"/>
@@ -3144,8 +3144,8 @@
       </c>
     </row>
     <row r="114" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B114" s="16"/>
-      <c r="C114" s="16"/>
+      <c r="B114" s="29"/>
+      <c r="C114" s="29"/>
       <c r="D114" s="6"/>
       <c r="E114" s="7"/>
       <c r="F114" s="6"/>
@@ -3159,8 +3159,8 @@
       </c>
     </row>
     <row r="115" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B115" s="16"/>
-      <c r="C115" s="16"/>
+      <c r="B115" s="29"/>
+      <c r="C115" s="29"/>
       <c r="D115" s="10"/>
       <c r="E115" s="11"/>
       <c r="F115" s="10"/>
@@ -3177,15 +3177,15 @@
       </c>
     </row>
     <row r="116" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B116" s="16"/>
-      <c r="C116" s="16"/>
+      <c r="B116" s="29"/>
+      <c r="C116" s="29"/>
       <c r="D116" s="6" t="s">
         <v>9</v>
       </c>
       <c r="E116" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="F116" s="18" t="s">
+      <c r="F116" s="26" t="s">
         <v>167</v>
       </c>
       <c r="G116" s="6" t="s">
@@ -3202,11 +3202,11 @@
       </c>
     </row>
     <row r="117" spans="2:11" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B117" s="26"/>
-      <c r="C117" s="26"/>
+      <c r="B117" s="20"/>
+      <c r="C117" s="20"/>
       <c r="D117" s="6"/>
       <c r="E117" s="7"/>
-      <c r="F117" s="18"/>
+      <c r="F117" s="26"/>
       <c r="G117" s="6"/>
       <c r="H117" s="6"/>
       <c r="I117" s="6" t="s">
@@ -3217,10 +3217,10 @@
       </c>
     </row>
     <row r="118" spans="2:11" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B118" s="26" t="s">
+      <c r="B118" s="20" t="s">
         <v>173</v>
       </c>
-      <c r="C118" s="26" t="s">
+      <c r="C118" s="20" t="s">
         <v>122</v>
       </c>
       <c r="D118" s="4" t="s">
@@ -3238,21 +3238,21 @@
       <c r="H118" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="I118" s="31" t="s">
+      <c r="I118" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="J118" s="31" t="s">
+      <c r="J118" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="K118" s="30" t="s">
+      <c r="K118" s="17" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="119" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B119" s="17"/>
-      <c r="C119" s="17"/>
+      <c r="B119" s="21"/>
+      <c r="C119" s="21"/>
       <c r="D119" s="6"/>
-      <c r="E119" s="20"/>
+      <c r="E119" s="24"/>
       <c r="F119" s="6"/>
       <c r="G119" s="6"/>
       <c r="H119" s="6"/>
@@ -3260,8 +3260,8 @@
       <c r="J119" s="6"/>
     </row>
     <row r="120" spans="2:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B120" s="17"/>
-      <c r="C120" s="17"/>
+      <c r="B120" s="21"/>
+      <c r="C120" s="21"/>
       <c r="D120" s="4" t="s">
         <v>51</v>
       </c>
@@ -3277,22 +3277,22 @@
       <c r="H120" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="I120" s="31" t="s">
+      <c r="I120" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="J120" s="31" t="s">
+      <c r="J120" s="18" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="121" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B121" s="17"/>
-      <c r="C121" s="17"/>
+      <c r="B121" s="21"/>
+      <c r="C121" s="21"/>
       <c r="D121" s="10"/>
       <c r="E121" s="15"/>
       <c r="F121" s="10"/>
       <c r="G121" s="10"/>
       <c r="H121" s="10"/>
-      <c r="I121" s="32" t="s">
+      <c r="I121" s="19" t="s">
         <v>28</v>
       </c>
       <c r="J121" s="10" t="s">
@@ -3300,8 +3300,8 @@
       </c>
     </row>
     <row r="122" spans="2:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B122" s="17"/>
-      <c r="C122" s="17" t="s">
+      <c r="B122" s="21"/>
+      <c r="C122" s="21" t="s">
         <v>154</v>
       </c>
       <c r="D122" s="6" t="s">
@@ -3319,31 +3319,31 @@
       <c r="H122" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="I122" s="29" t="s">
+      <c r="I122" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="J122" s="29" t="s">
+      <c r="J122" s="16" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="123" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B123" s="17"/>
-      <c r="C123" s="17"/>
+      <c r="B123" s="21"/>
+      <c r="C123" s="21"/>
       <c r="D123" s="6"/>
       <c r="E123" s="7"/>
       <c r="F123" s="6"/>
       <c r="G123" s="6"/>
       <c r="H123" s="6"/>
-      <c r="I123" s="29" t="s">
+      <c r="I123" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="J123" s="29" t="s">
+      <c r="J123" s="16" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="124" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B124" s="17"/>
-      <c r="C124" s="17"/>
+      <c r="B124" s="21"/>
+      <c r="C124" s="21"/>
       <c r="D124" s="6"/>
       <c r="E124" s="7"/>
       <c r="F124" s="6"/>
@@ -3353,8 +3353,8 @@
       <c r="J124" s="6"/>
     </row>
     <row r="125" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B125" s="17"/>
-      <c r="C125" s="17"/>
+      <c r="B125" s="21"/>
+      <c r="C125" s="21"/>
       <c r="D125" s="6"/>
       <c r="E125" s="7"/>
       <c r="F125" s="6"/>
@@ -3364,8 +3364,8 @@
       <c r="J125" s="6"/>
     </row>
     <row r="126" spans="2:11" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B126" s="17"/>
-      <c r="C126" s="18" t="s">
+      <c r="B126" s="21"/>
+      <c r="C126" s="26" t="s">
         <v>59</v>
       </c>
       <c r="D126" s="4" t="s">
@@ -3374,7 +3374,7 @@
       <c r="E126" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="F126" s="21" t="s">
+      <c r="F126" s="25" t="s">
         <v>182</v>
       </c>
       <c r="G126" s="4" t="s">
@@ -3383,31 +3383,31 @@
       <c r="H126" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="I126" s="31" t="s">
+      <c r="I126" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="J126" s="31" t="s">
+      <c r="J126" s="18" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="127" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B127" s="17"/>
-      <c r="C127" s="18"/>
+      <c r="B127" s="21"/>
+      <c r="C127" s="26"/>
       <c r="D127" s="6"/>
       <c r="E127" s="7"/>
-      <c r="F127" s="18"/>
+      <c r="F127" s="26"/>
       <c r="G127" s="6"/>
       <c r="H127" s="6"/>
-      <c r="I127" s="29" t="s">
+      <c r="I127" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="J127" s="29" t="s">
+      <c r="J127" s="16" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="128" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B128" s="27"/>
-      <c r="C128" s="19"/>
+      <c r="B128" s="22"/>
+      <c r="C128" s="27"/>
       <c r="D128" s="10"/>
       <c r="E128" s="11"/>
       <c r="F128" s="10"/>
@@ -3423,12 +3423,30 @@
     <row r="129" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="46">
-    <mergeCell ref="B118:B128"/>
-    <mergeCell ref="E118:E119"/>
-    <mergeCell ref="F126:F127"/>
-    <mergeCell ref="C118:C121"/>
-    <mergeCell ref="C122:C125"/>
-    <mergeCell ref="C126:C128"/>
+    <mergeCell ref="B82:B92"/>
+    <mergeCell ref="G95:G96"/>
+    <mergeCell ref="G103:G104"/>
+    <mergeCell ref="F82:F83"/>
+    <mergeCell ref="C106:C117"/>
+    <mergeCell ref="B101:B117"/>
+    <mergeCell ref="F106:F108"/>
+    <mergeCell ref="F116:F117"/>
+    <mergeCell ref="B93:B100"/>
+    <mergeCell ref="E95:E97"/>
+    <mergeCell ref="C101:C105"/>
+    <mergeCell ref="C93:C100"/>
+    <mergeCell ref="G56:G57"/>
+    <mergeCell ref="G77:G79"/>
+    <mergeCell ref="G80:G81"/>
+    <mergeCell ref="G84:G85"/>
+    <mergeCell ref="C82:C92"/>
+    <mergeCell ref="C77:C81"/>
+    <mergeCell ref="B71:B81"/>
+    <mergeCell ref="F74:F76"/>
+    <mergeCell ref="C71:C76"/>
+    <mergeCell ref="F71:F73"/>
+    <mergeCell ref="E77:E79"/>
+    <mergeCell ref="E80:E81"/>
     <mergeCell ref="B22:B37"/>
     <mergeCell ref="E63:E64"/>
     <mergeCell ref="G11:G13"/>
@@ -3445,30 +3463,12 @@
     <mergeCell ref="F56:F57"/>
     <mergeCell ref="C38:C55"/>
     <mergeCell ref="C56:C70"/>
-    <mergeCell ref="C77:C81"/>
-    <mergeCell ref="B71:B81"/>
-    <mergeCell ref="F74:F76"/>
-    <mergeCell ref="C71:C76"/>
-    <mergeCell ref="F71:F73"/>
-    <mergeCell ref="E77:E79"/>
-    <mergeCell ref="E80:E81"/>
-    <mergeCell ref="C93:C100"/>
-    <mergeCell ref="G56:G57"/>
-    <mergeCell ref="G77:G79"/>
-    <mergeCell ref="G80:G81"/>
-    <mergeCell ref="G84:G85"/>
-    <mergeCell ref="C82:C92"/>
-    <mergeCell ref="B82:B92"/>
-    <mergeCell ref="G95:G96"/>
-    <mergeCell ref="G103:G104"/>
-    <mergeCell ref="F82:F83"/>
-    <mergeCell ref="C106:C117"/>
-    <mergeCell ref="B101:B117"/>
-    <mergeCell ref="F106:F108"/>
-    <mergeCell ref="F116:F117"/>
-    <mergeCell ref="B93:B100"/>
-    <mergeCell ref="E95:E97"/>
-    <mergeCell ref="C101:C105"/>
+    <mergeCell ref="B118:B128"/>
+    <mergeCell ref="E118:E119"/>
+    <mergeCell ref="F126:F127"/>
+    <mergeCell ref="C118:C121"/>
+    <mergeCell ref="C122:C125"/>
+    <mergeCell ref="C126:C128"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>